<commit_message>
feat: optimizacion de ROSI y adicionalmente ajustes en evaluator para correcto funcionamiento de la shiny app
</commit_message>
<xml_diff>
--- a/app/evaluator_workspace/inputs/survey.xlsx
+++ b/app/evaluator_workspace/inputs/survey.xlsx
@@ -23,6 +23,7 @@
     <sheet name="IM" sheetId="20" state="visible" r:id="rId15"/>
     <sheet name="BC" sheetId="17" state="visible" r:id="rId16"/>
     <sheet name="PRI" sheetId="5" state="visible" r:id="rId17"/>
+    <sheet name="SINPE" sheetId="22" state="visible" r:id="rId18"/>
   </sheets>
   <definedNames>
     <definedName name="DIFF_Values">Reference!$A$17:$A$21</definedName>
@@ -35,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="346" uniqueCount="346">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="692" uniqueCount="692">
   <si>
     <t>Threats</t>
   </si>
@@ -1073,6 +1074,1044 @@
   </si>
   <si>
     <t xml:space="preserve">CAP-01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Marco de seguridad de la información institucional</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2 - Repetible</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Personal de seguridad de la información capacitado</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Roles y responsabilidades de seguridad claramente definidos</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3 - Definido</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Verificación de identidad y registro de usuarios</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Gestión del ciclo de vida de cuentas de usuario y sistema</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Divulgación comunitaria y colaboración con otras organizaciones</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Programa de concientización y educación en seguridad y privacidad</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Revisión de contenido y educación en políticas de seguridad</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1 - Inicial</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Comunicación de responsabilidades de seguridad al personal</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Programa de identificación y tratamiento de riesgos</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Aceptación de riesgos residuales por los propietarios del riesgo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Evaluaciones de riesgo en aplicaciones, sistemas y redes críticas</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5 - Optimizado</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Reporte de condiciones de riesgo a la alta dirección</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Defensoría de disputas y quejas sobre políticas de seguridad</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Monitoreo de autoridades externas y tendencias de la industria</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Documentación y revisión de incumplimientos de políticas</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Políticas de seguridad alineadas a requisitos de negocio y legales</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Comité directivo de supervisión de privacidad y seguridad de la información</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Autoridad delegada para la respuesta a incidentes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Coordinación de actividades de seguridad entre departamentos</t>
+  </si>
+  <si>
+    <t xml:space="preserve">4 - Gestionado</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Estrategia y compromiso de la alta dirección en seguridad</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Programa de inteligencia activa</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Autoevaluación periódica del programa de seguridad</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Verificación periódica de los controles de seguridad</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Verificación de controles de terceros con acceso a información confidencial</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cumplimiento de requisitos de negocio y privacidad</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Revisión periódica del cumplimiento en sistemas críticos</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Inventario, clasificación y propiedad de la información</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Manejo y destrucción de medios y dispositivos</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Control de acceso físico a instalaciones críticas</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Protección física de instalaciones críticas</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Protección física de sistemas críticos e información institucional</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Plan de seguridad física</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Gestión de cambios y configuración</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Estándar de uso aceptable</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Estándares de construcción y mantenimiento de hardware y software</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Estándares de arquitectura técnica de seguridad y privacidad</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cifrado y protección de datos en tránsito y en reposo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Gestión de acceso remoto y externo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Proceso de autorización de acceso de usuarios y sistemas</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Autenticación de usuarios y sistemas (incluye MFA)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Segmentación y protección de red, sistemas y aplicaciones</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Proceso de destrucción o eliminación segura de datos</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Medición de referencia de actividad en aplicaciones, sistemas y redes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Detección de intrusiones</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Registro de actividad de redes, sistemas y aplicaciones</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Monitoreo de sistemas críticos</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Gestión de vulnerabilidades y remediación de fallas</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ciclo de vida de desarrollo seguro de aplicaciones</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Proceso de gestión de incidentes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Relaciones con terceros y expertos en respuesta a incidentes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Capacidades de investigación forense</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Identificación, respuesta, mitigación y documentación de incidentes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Proceso de retención legal de información</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Planes de continuidad del negocio y recuperación ante desastres</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Proceso sistemático de respaldo de información crítica</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Política de privacidad en línea y términos de uso</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Controles de seguridad y responsabilidad de la privacidad</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Minimización, anonimización y eliminación de información confidencial</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Programa de privacidad coordinado con el Oficial de Privacidad</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dificultad (DIFF) - Nivel de Madurez del Control (CMM)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Optimizado. Completamente efectivo. De clase mundial.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Probado y revisado.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Se considera práctica estándar y operativa.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Repetible y posiblemente consistente en toda la organización.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">No se realiza o se realiza de forma inconsistente.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Capacidad de Amenaza (TC) - Capacidad de la Comunidad de Amenazas</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Alto</t>
+  </si>
+  <si>
+    <t xml:space="preserve">El actor es extremadamente capaz (de clase mundial).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Medio</t>
+  </si>
+  <si>
+    <t xml:space="preserve">El actor de amenazas tiene capacidad típica.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bajo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">El actor de amenazas tiene baja capacidad.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Frecuencia Esperada de Amenazas (TEF) - Ocurrencia de Amenazas Contra el Control</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Frecuente</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Oportunidades de materialización muchas veces al mes.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ocasional</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Oportunidades de materialización varias veces al año.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Raro</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Oportunidades de materialización menos de una vez al año.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Magnitud de Pérdida (LM) - Tamaño de la Pérdida si el Escenario Ocurre</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Alta</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Efecto real y serio en resultados y/o capacidad de generar ingresos a largo plazo.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Media</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Efecto significativo en la utilidad anual.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Baja</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Absorbida por las actividades normales.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Frecuencia de Eventos de Amenaza (TEF)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Capacidad de Amenaza (TC)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Magnitud de Pérdida (LM)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dificultad del Control (DIFF)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Acceso no autorizado a información confidencial de clientes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ciberdelincuentes externos</t>
+  </si>
+  <si>
+    <t xml:space="preserve">dist:pert|params:min=2,mode=6,max=15</t>
+  </si>
+  <si>
+    <t xml:space="preserve">dist:pert|params:min=0.5,mode=0.75,max=0.98</t>
+  </si>
+  <si>
+    <t xml:space="preserve">dist:pert|params:min=500000,mode=2000000,max=8000000</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RS-001</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CAP-02, CAP-49, CAP-50</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Filtración de datos de clientes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ciberdelincuentes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Escenario de verificación final</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Insiders</t>
+  </si>
+  <si>
+    <t xml:space="preserve">dist:pert|params:min=1,mode=4,max=10</t>
+  </si>
+  <si>
+    <t xml:space="preserve">dist:pert|params:min=0.3,mode=0.6,max=0.9</t>
+  </si>
+  <si>
+    <t xml:space="preserve">dist:pert|params:min=100000,mode=1000000,max=5000000</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RS-VERIF</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CAP-49</t>
+  </si>
+  <si>
+    <t xml:space="preserve">prueba</t>
+  </si>
+  <si>
+    <t xml:space="preserve">afr0</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Frequent</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Medium</t>
+  </si>
+  <si>
+    <t xml:space="preserve"/>
+  </si>
+  <si>
+    <t xml:space="preserve">Prueba importacion CSV</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RS-X</t>
+  </si>
+  <si>
+    <t xml:space="preserve">frequent</t>
+  </si>
+  <si>
+    <t xml:space="preserve">medium</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Acceso no autorizado desde el exterior</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hacktivistas</t>
+  </si>
+  <si>
+    <t xml:space="preserve">high</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SEC-001</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CAP-49, CAP-50</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fuga de datos de clientes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">IMP-001</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CAP-46, CAP-49</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ransomware en servidores</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Grupos de ransomware</t>
+  </si>
+  <si>
+    <t xml:space="preserve">occasional</t>
+  </si>
+  <si>
+    <t xml:space="preserve">IMP-002</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CAP-41, CAP-50</t>
+  </si>
+  <si>
+    <t xml:space="preserve">dist:lnorm;params:meanlog=8.064, sdlog=1.526</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Inadequate human resources are available to execute the informaton security strategic security plan.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Technology Leadership</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RS-01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CAP-01, CAP-05, CAP-07, CAP-32, CAP-14, CAP-15, CAP-16</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Budget does not adequately support the information security strategic plan.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RS-02</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Competing priorities within the institution results in inability to execute the information security strategic security plan.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RS-03</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Increased negligence by workforce members due to lack of appropriate delegated authority and security support.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RS-04</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CAP-01, CAP-03, CAP-05, CAP-07, CAP-32, CAP-14, CAP-15, CAP-16</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The information security function implements a strategy that has unanticipated consequences on the insitution, interfering with other stated business objectives.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">low</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RS-05</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CAP-01, CAP-07, CAP-14, CAP-15, CAP-16</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Inconsistent interpretation or insecure actions by workforce.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Organizational Internal Users</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RS-06</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CAP-09, CAP-10, CAP-11, CAP-12</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Misuse of information assets.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RS-07</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Noncompliance with laws, regulations, and contractual agreements.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">rare</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RS-08</t>
+  </si>
+  <si>
+    <t xml:space="preserve">New or changing privacy regulations are not implemented in organizational IT systems.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Regulators or Auditors</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RS-09</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CAP-08, CAP-13</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Internal workforce members execute financial fraud, embezzlement, or information theft made possible through lack of internal controls.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RS-10</t>
+  </si>
+  <si>
+    <t xml:space="preserve">External attackers locate previously unknown weaknesses in the information security program not revealed through internal controls.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">External Cyber Adversaries</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RS-11</t>
+  </si>
+  <si>
+    <t xml:space="preserve">External auditors find compliance issues with regulations and standards not identified via internal processes.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RS-12</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Inability to accurately forecast the consequences of adopted technologies or innovations.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RS-13</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CAP-17, CAP-18, CAP-19, CAP-20</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lack of risk management at leadership level results in inability to adjust strategic and tactical plans to changing external threat environment.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RS-14</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Inability to understand specific threats related to attackers.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RS-15</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Security failure or instability of providers or partners results in disclosure of organizational data.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RS-16</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Internal user inappropriate use or misuse of information.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RS-17</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CAP-21, CAP-22, CAP-23, CAP-24</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Systemic noncompliance with privacy laws, regulations, and contractual agreements.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RS-18</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Organizational security team cannot identify nor correct root cause of information breach, resulting in rework.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RS-19</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CAP-25, CAP-26, CAP-27, CAP-28, CAP-59</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lack of incident handling results in noncompliance with laws, regulations, and contractual agreements.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RS-20</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Failure to address security incidents results in reputation loss.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RS-21</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Undetected and unremediated security incidents result in unmitigated access.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RS-22</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Inadequate investigation results in inappropriate notifications.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RS-23</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Changing cultural norms on the use of data combined with insufficient education results in privacy violations.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RS-24</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CAP-30, CAP-31, CAP-60</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Through insufficient training, workforce members cannot identify (or fail to report) potential information security incidents, resulting in loss from undetected attacks.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RS-25</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CAP-29, CAP-30, CAP-31, CAP-60</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Misuse of information assets or user errors (data entry errors, omissions, inadvertent acts or carelessness).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RS-26</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Successful social engineering attacks result in information or financial loss.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RS-27</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Unknown attack intelligence results in undetected events.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RS-28</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CAP-33, CAP-34, CAP-35, CAP-36</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Unknown incidence of security breach</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RS-29</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lack of monitoring demonstrates failure to take due care, resulting in non-compliance with associated laws and regulations.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RS-30</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Business disruption and non-recovery of data.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RS-31</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CAP-41, CAP-45</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Changing or adding software without authorization results in system performance or data disclosure.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RS-32</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CAP-37, CAP-38, CAP-40, CAP-41, CAP-42, CAP-43, CAP-46, CAP-47, CAP-48, CAP-49, CAP-50, CAP-39, CAP-51, CAP-33, CAP-34, CAP-35, CAP-36</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Malfunction of business application and system software.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RS-33</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lack of ability to respond to targeted malware (Trojan horse, spyware, BOTS, worms, and viruses) results in compromise of data assets.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RS-34</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Breach through technical controls results in reportable significant unauthorized disclosure of data.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RS-35</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Unforeseen effect of changes to software, computer, and communications equipment.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RS-36</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Destruction, misuse, or modification of information assets through breach of technical controls.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RS-37</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Eroding network boundaries result in lack of defenses on systems.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RS-38</t>
+  </si>
+  <si>
+    <t xml:space="preserve">External attackers breach technical controls and gain unauthorized access to systems and networks.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RS-39</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Unintended consequence of implemented information security controls on workforce or connected devices.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RS-40</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Damage to or loss of information systems and network services through terror-related physical attack.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Political Activists</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RS-41</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CAP-52, CAP-53, CAP-54, CAP-55</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Damage to or loss of physical facility through natural disaster.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Environmental</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RS-42</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Inappropriate release of information assets through physical disclosure.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RS-43</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Theft or loss of physical assets.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RS-44</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Loss of information assets due to misclassification and non-classification.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RS-45</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CAP-56, CAP-39</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Misclassification due to data aggregation.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RS-46</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lack of accountability for critical information and systems results in inappropriate control and inventory.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RS-47</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Unauthorized access to or use of information and systems results in inappropriate use by internal users.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RS-48</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CAP-57, CAP-58</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Uncontrolled aggregation, proliferation, and use of data.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RS-49</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Inadequate response results in inappropriate internal use of data.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RS-50</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Unauthorized access to or use of information and systems.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Third Parties</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RS-51</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Inability to respond to litgation holds.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">External Litigants</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RS-52</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CAP-59</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Inability to respond to HR investigations results in avoidable adverse judgements.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RS-53</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Damage to or loss of information system due to natural disaster at physical facility.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RS-55</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RS-56</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CAP-38, CAP-44</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Prueba control personalizado</t>
+  </si>
+  <si>
+    <t xml:space="preserve">dist:pert|params:min=2,mode=5,max=12</t>
+  </si>
+  <si>
+    <t xml:space="preserve">dist:pert|params:min=0.4,mode=0.7,max=0.95</t>
+  </si>
+  <si>
+    <t xml:space="preserve">dist:pert|params:min=100000,mode=800000,max=3000000</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RS-CUSTOM</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CAP-99</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Capabilities</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Name</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DIFF</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Evidence</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CapabilityID</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Threats</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Scenario</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TComm</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TEF</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LM</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ScenarioID</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Exfiltración de datos personales</t>
+  </si>
+  <si>
+    <t xml:space="preserve">dist:pert|params:min=200000,mode=1000000,max=5000000</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GDPR-01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CTRL-01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">High</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RS-9999</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CTRL-01, CTRL-02</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Acceso no autorizado a datos de clientes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RS-900</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CTRL-03</t>
+  </si>
+  <si>
+    <t xml:space="preserve">prueba 3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">prueba 4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RS-777</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RS-7</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Filtración de datos personales</t>
+  </si>
+  <si>
+    <t xml:space="preserve">pruena 2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Segmento 1 SINPE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">dist:pert|params:min=1006.54,mode=5959.39,max=11680.36</t>
+  </si>
+  <si>
+    <t xml:space="preserve">dist:pert|params:min=0.21,mode=0.5,max=0.79</t>
+  </si>
+  <si>
+    <t xml:space="preserve">dist:gamma|params:</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SINPE-1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CTRL-03, CTRL-04, CTRL-05, CTRL-06, CTRL-07, CTRL-08</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Exfiltración</t>
+  </si>
+  <si>
+    <t xml:space="preserve">dist:lnorm|params:meanlog=1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NO-EXISTE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fuga por correo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DLP-01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SINPE segmento 1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ciber delincuentes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">dist:lnorm|params:meanlog=2.681, sdlog=3.128</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ciber delincuente</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SINPE del Segmento 1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SINPE-001</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CTRL-0101, CTRL-0102, CTRL-0103, CTRL-0104, CTRL-0105, CTRL-0106</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SINPE del Segmento 2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[Requiere datos de saldos para ajuste]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SINPE-002</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CTRL-0201, CTRL-0202, CTRL-0203, CTRL-0204, CTRL-0205, CTRL-0206</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SINPE del Segmento 3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SINPE-003</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CTRL-0301, CTRL-0302, CTRL-0303, CTRL-0304, CTRL-0305, CTRL-0306</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SINPE del Segmento 4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SINPE-004</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CTRL-0401, CTRL-0402, CTRL-0403, CTRL-0404, CTRL-0405, CTRL-0406</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SINPE del Segmento 5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SINPE-005</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CTRL-0501, CTRL-0502, CTRL-0503, CTRL-0504, CTRL-0505, CTRL-0506</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SINPE del Segmento 6</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SINPE-006</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CTRL-0601, CTRL-0602, CTRL-0603, CTRL-0604, CTRL-0605, CTRL-0606</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SINPE del Segmento 7</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SINPE-007</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CTRL-0701, CTRL-0702, CTRL-0703, CTRL-0704, CTRL-0705, CTRL-0706</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SINPE del Segmento 8</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SINPE-008</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CTRL-0801, CTRL-0802, CTRL-0803, CTRL-0804, CTRL-0805, CTRL-0806</t>
   </si>
 </sst>
 </file>
@@ -1685,65 +2724,7 @@
 </file>
 
 <file path=xl/tables/table10.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="10" xr:uid="{00000000-000C-0000-FFFF-FFFF08000000}" name="AC_Threats" displayName="AC_Threats" ref="A7:G9" totalsRowShown="0" headerRowDxfId="69" headerRowBorderDxfId="68" tableBorderDxfId="67">
-  <autoFilter ref="A7:G9" xr:uid="{00000000-0009-0000-0100-00001B000000}"/>
-  <tableColumns count="7">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0800-000001000000}" name="Scenario" dataDxfId="66"/>
-    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0800-000007000000}" name="TComm" dataDxfId="65"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0800-000002000000}" name="TEF"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0800-000003000000}" name="TC"/>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0800-000004000000}" name="LM"/>
-    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0800-000006000000}" name="ScenarioID"/>
-    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0800-000005000000}" name="Capabilities"/>
-  </tableColumns>
-  <tableStyleInfo name="TableStyleLight2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
-</table>
-</file>
-
-<file path=xl/tables/table11.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="11" xr:uid="{00000000-000C-0000-FFFF-FFFF07000000}" name="AC_Capabilities" displayName="AC_Capabilities" ref="A2:D4" totalsRowShown="0" headerRowDxfId="73" headerRowBorderDxfId="72" tableBorderDxfId="71">
-  <autoFilter ref="A2:D4" xr:uid="{00000000-0009-0000-0100-000004000000}"/>
-  <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0700-000001000000}" name="Name" dataDxfId="70"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0700-000002000000}" name="DIFF"/>
-    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0700-000005000000}" name="Evidence"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0700-000003000000}" name="CapabilityID"/>
-  </tableColumns>
-  <tableStyleInfo name="TableStyleLight2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
-</table>
-</file>
-
-<file path=xl/tables/table12.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="12" xr:uid="{00000000-000C-0000-FFFF-FFFF0A000000}" name="HR_Threats" displayName="HR_Threats" ref="A9:G13" totalsRowShown="0">
-  <autoFilter ref="A9:G13" xr:uid="{00000000-0009-0000-0100-000014000000}"/>
-  <tableColumns count="7">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0A00-000001000000}" name="Scenario" dataDxfId="60"/>
-    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0A00-000007000000}" name="TComm" dataDxfId="59"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0A00-000002000000}" name="TEF"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0A00-000003000000}" name="TC"/>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0A00-000004000000}" name="LM"/>
-    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0A00-000006000000}" name="ScenarioID"/>
-    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0A00-000005000000}" name="Capabilities"/>
-  </tableColumns>
-  <tableStyleInfo name="TableStyleLight2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
-</table>
-</file>
-
-<file path=xl/tables/table13.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="13" xr:uid="{00000000-000C-0000-FFFF-FFFF09000000}" name="HR_Capabilites" displayName="HR_Capabilites" ref="A2:D6" totalsRowShown="0" headerRowDxfId="64" headerRowBorderDxfId="63" tableBorderDxfId="62">
-  <autoFilter ref="A2:D6" xr:uid="{00000000-0009-0000-0100-00000A000000}"/>
-  <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0900-000001000000}" name="Name" dataDxfId="61"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0900-000002000000}" name="DIFF"/>
-    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0900-000005000000}" name="Evidence"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0900-000003000000}" name="CapabilityID"/>
-  </tableColumns>
-  <tableStyleInfo name="TableStyleLight2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
-</table>
-</file>
-
-<file path=xl/tables/table14.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="14" xr:uid="{00000000-000C-0000-FFFF-FFFF0C000000}" name="Risk_Threats" displayName="Risk_Threats" ref="A9:G13" totalsRowShown="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="10" xr:uid="{00000000-000C-0000-FFFF-FFFF0C000000}" name="Risk_Threats" displayName="Risk_Threats" ref="A9:G13" totalsRowShown="0">
   <autoFilter ref="A9:G13" xr:uid="{00000000-0009-0000-0100-000017000000}"/>
   <tableColumns count="7">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0C00-000001000000}" name="Scenario" dataDxfId="54"/>
@@ -1758,8 +2739,8 @@
 </table>
 </file>
 
-<file path=xl/tables/table15.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="15" xr:uid="{00000000-000C-0000-FFFF-FFFF0B000000}" name="Risk_Capabilities" displayName="Risk_Capabilities" ref="A2:D6" totalsRowShown="0" headerRowDxfId="58" headerRowBorderDxfId="57" tableBorderDxfId="56">
+<file path=xl/tables/table11.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="11" xr:uid="{00000000-000C-0000-FFFF-FFFF0B000000}" name="Risk_Capabilities" displayName="Risk_Capabilities" ref="A2:D6" totalsRowShown="0" headerRowDxfId="58" headerRowBorderDxfId="57" tableBorderDxfId="56">
   <autoFilter ref="A2:D6" xr:uid="{00000000-0009-0000-0100-00000D000000}"/>
   <tableColumns count="4">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0B00-000001000000}" name="Name" dataDxfId="55"/>
@@ -1771,8 +2752,8 @@
 </table>
 </file>
 
-<file path=xl/tables/table16.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="16" xr:uid="{00000000-000C-0000-FFFF-FFFF0E000000}" name="Policy_Capabilities" displayName="Policy_Capabilities" ref="A2:D6" totalsRowShown="0" headerRowDxfId="50" headerRowBorderDxfId="49" tableBorderDxfId="48">
+<file path=xl/tables/table12.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="12" xr:uid="{00000000-000C-0000-FFFF-FFFF0E000000}" name="Policy_Capabilities" displayName="Policy_Capabilities" ref="A2:D6" totalsRowShown="0" headerRowDxfId="50" headerRowBorderDxfId="49" tableBorderDxfId="48">
   <autoFilter ref="A2:D6" xr:uid="{00000000-0009-0000-0100-00000F000000}"/>
   <tableColumns count="4">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0E00-000001000000}" name="Name" dataDxfId="47"/>
@@ -1784,8 +2765,8 @@
 </table>
 </file>
 
-<file path=xl/tables/table17.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="17" xr:uid="{00000000-000C-0000-FFFF-FFFF0D000000}" name="Policy_Threats" displayName="Policy_Threats" ref="A9:G12" totalsRowShown="0">
+<file path=xl/tables/table13.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="13" xr:uid="{00000000-000C-0000-FFFF-FFFF0D000000}" name="Policy_Threats" displayName="Policy_Threats" ref="A9:G12" totalsRowShown="0">
   <autoFilter ref="A9:G12" xr:uid="{00000000-0009-0000-0100-000019000000}"/>
   <tableColumns count="7">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0D00-000001000000}" name="Scenario" dataDxfId="52"/>
@@ -1800,8 +2781,8 @@
 </table>
 </file>
 
-<file path=xl/tables/table18.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="18" xr:uid="{00000000-000C-0000-FFFF-FFFF10000000}" name="ORG_Threats" displayName="ORG_Threats" ref="A13:G18" totalsRowShown="0">
+<file path=xl/tables/table14.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="14" xr:uid="{00000000-000C-0000-FFFF-FFFF10000000}" name="ORG_Threats" displayName="ORG_Threats" ref="A13:G18" totalsRowShown="0">
   <autoFilter ref="A13:G18" xr:uid="{00000000-0009-0000-0100-000012000000}"/>
   <tableColumns count="7">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-1000-000001000000}" name="Scenario" dataDxfId="45"/>
@@ -1816,8 +2797,8 @@
 </table>
 </file>
 
-<file path=xl/tables/table19.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="19" xr:uid="{00000000-000C-0000-FFFF-FFFF0F000000}" name="ORG_Capabilities" displayName="ORG_Capabilities" ref="A2:D10" totalsRowShown="0">
+<file path=xl/tables/table15.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="15" xr:uid="{00000000-000C-0000-FFFF-FFFF0F000000}" name="ORG_Capabilities" displayName="ORG_Capabilities" ref="A2:D10" totalsRowShown="0">
   <autoFilter ref="A2:D10" xr:uid="{00000000-0009-0000-0100-000011000000}"/>
   <tableColumns count="4">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0F00-000001000000}" name="Name" dataDxfId="46"/>
@@ -1829,8 +2810,8 @@
 </table>
 </file>
 
-<file path=xl/tables/table20.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="20" xr:uid="{00000000-000C-0000-FFFF-FFFF12000000}" name="COMP_Threats" displayName="COMP_Threats" ref="A7:G11" totalsRowShown="0">
+<file path=xl/tables/table16.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="16" xr:uid="{00000000-000C-0000-FFFF-FFFF12000000}" name="COMP_Threats" displayName="COMP_Threats" ref="A7:G11" totalsRowShown="0">
   <autoFilter ref="A7:G11" xr:uid="{00000000-0009-0000-0100-000018000000}"/>
   <tableColumns count="7">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-1200-000001000000}" name="Scenario" dataDxfId="40"/>
@@ -1845,8 +2826,8 @@
 </table>
 </file>
 
-<file path=xl/tables/table21.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="21" xr:uid="{00000000-000C-0000-FFFF-FFFF11000000}" name="COMP_Capabilities" displayName="COMP_Capabilities" ref="A2:D4" totalsRowShown="0">
+<file path=xl/tables/table17.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="17" xr:uid="{00000000-000C-0000-FFFF-FFFF11000000}" name="COMP_Capabilities" displayName="COMP_Capabilities" ref="A2:D4" totalsRowShown="0">
   <autoFilter ref="A2:D4" xr:uid="{00000000-0009-0000-0100-00000E000000}"/>
   <tableColumns count="4">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-1100-000001000000}" name="Name" dataDxfId="42"/>
@@ -1858,8 +2839,8 @@
 </table>
 </file>
 
-<file path=xl/tables/table22.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="22" xr:uid="{00000000-000C-0000-FFFF-FFFF14000000}" name="Asset_Threats" displayName="Asset_Threats" ref="A7:G10" totalsRowShown="0" headerRowDxfId="34" headerRowBorderDxfId="33" tableBorderDxfId="32">
+<file path=xl/tables/table18.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="18" xr:uid="{00000000-000C-0000-FFFF-FFFF14000000}" name="Asset_Threats" displayName="Asset_Threats" ref="A7:G10" totalsRowShown="0" headerRowDxfId="34" headerRowBorderDxfId="33" tableBorderDxfId="32">
   <autoFilter ref="A7:G10" xr:uid="{00000000-0009-0000-0100-00001A000000}"/>
   <tableColumns count="7">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-1400-000001000000}" name="Scenario" dataDxfId="31"/>
@@ -1874,8 +2855,8 @@
 </table>
 </file>
 
-<file path=xl/tables/table23.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="23" xr:uid="{00000000-000C-0000-FFFF-FFFF13000000}" name="Asset_Capabilities" displayName="Asset_Capabilities" ref="A2:D4" totalsRowShown="0" headerRowDxfId="38" headerRowBorderDxfId="37" tableBorderDxfId="36">
+<file path=xl/tables/table19.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="19" xr:uid="{00000000-000C-0000-FFFF-FFFF13000000}" name="Asset_Capabilities" displayName="Asset_Capabilities" ref="A2:D4" totalsRowShown="0" headerRowDxfId="38" headerRowBorderDxfId="37" tableBorderDxfId="36">
   <autoFilter ref="A2:D4" xr:uid="{00000000-0009-0000-0100-000005000000}"/>
   <tableColumns count="4">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-1300-000001000000}" name="Name" dataDxfId="35"/>
@@ -1887,8 +2868,8 @@
 </table>
 </file>
 
-<file path=xl/tables/table24.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="24" xr:uid="{00000000-000C-0000-FFFF-FFFF16000000}" name="Physical_Threats" displayName="Physical_Threats" ref="A9:G13" totalsRowShown="0">
+<file path=xl/tables/table20.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="20" xr:uid="{00000000-000C-0000-FFFF-FFFF16000000}" name="Physical_Threats" displayName="Physical_Threats" ref="A9:G13" totalsRowShown="0">
   <autoFilter ref="A9:G13" xr:uid="{00000000-0009-0000-0100-000010000000}"/>
   <tableColumns count="7">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-1600-000001000000}" name="Scenario" dataDxfId="28"/>
@@ -1903,8 +2884,8 @@
 </table>
 </file>
 
-<file path=xl/tables/table25.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="25" xr:uid="{00000000-000C-0000-FFFF-FFFF15000000}" name="Physical_Capabilities" displayName="Physical_Capabilities" ref="A2:D6" totalsRowShown="0">
+<file path=xl/tables/table21.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="21" xr:uid="{00000000-000C-0000-FFFF-FFFF15000000}" name="Physical_Capabilities" displayName="Physical_Capabilities" ref="A2:D6" totalsRowShown="0">
   <autoFilter ref="A2:D6" xr:uid="{00000000-0009-0000-0100-000006000000}"/>
   <tableColumns count="4">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-1500-000001000000}" name="Name" dataDxfId="29"/>
@@ -1916,8 +2897,8 @@
 </table>
 </file>
 
-<file path=xl/tables/table26.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="26" xr:uid="{00000000-000C-0000-FFFF-FFFF18000000}" name="OPS_Threats" displayName="OPS_Threats" ref="A19:G27" totalsRowShown="0">
+<file path=xl/tables/table22.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="22" xr:uid="{00000000-000C-0000-FFFF-FFFF18000000}" name="OPS_Threats" displayName="OPS_Threats" ref="A19:G27" totalsRowShown="0">
   <autoFilter ref="A19:G27" xr:uid="{00000000-0009-0000-0100-00001F000000}"/>
   <tableColumns count="7">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-1800-000001000000}" name="Scenario" dataDxfId="25"/>
@@ -1932,8 +2913,8 @@
 </table>
 </file>
 
-<file path=xl/tables/table27.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="27" xr:uid="{00000000-000C-0000-FFFF-FFFF17000000}" name="OPS_Capabilities" displayName="OPS_Capabilities" ref="A2:D16" totalsRowShown="0">
+<file path=xl/tables/table23.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="23" xr:uid="{00000000-000C-0000-FFFF-FFFF17000000}" name="OPS_Capabilities" displayName="OPS_Capabilities" ref="A2:D16" totalsRowShown="0">
   <autoFilter ref="A2:D16" xr:uid="{00000000-0009-0000-0100-00001E000000}"/>
   <tableColumns count="4">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-1700-000001000000}" name="Name" dataDxfId="26"/>
@@ -1945,8 +2926,8 @@
 </table>
 </file>
 
-<file path=xl/tables/table28.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="28" xr:uid="{00000000-000C-0000-FFFF-FFFF1A000000}" name="ADM_Threats" displayName="ADM_Threats" ref="A7:G8" totalsRowShown="0">
+<file path=xl/tables/table24.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="24" xr:uid="{00000000-000C-0000-FFFF-FFFF1A000000}" name="ADM_Threats" displayName="ADM_Threats" ref="A7:G8" totalsRowShown="0">
   <autoFilter ref="A7:G8" xr:uid="{00000000-0009-0000-0100-000015000000}"/>
   <tableColumns count="7">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-1A00-000001000000}" name="Scenario" dataDxfId="21"/>
@@ -1961,14 +2942,72 @@
 </table>
 </file>
 
-<file path=xl/tables/table29.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="29" xr:uid="{00000000-000C-0000-FFFF-FFFF19000000}" name="ADM_Capabilities" displayName="ADM_Capabilities" ref="A2:D4" totalsRowShown="0">
+<file path=xl/tables/table25.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="25" xr:uid="{00000000-000C-0000-FFFF-FFFF19000000}" name="ADM_Capabilities" displayName="ADM_Capabilities" ref="A2:D4" totalsRowShown="0">
   <autoFilter ref="A2:D4" xr:uid="{00000000-0009-0000-0100-000013000000}"/>
   <tableColumns count="4">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-1900-000001000000}" name="Name" dataDxfId="22"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-1900-000002000000}" name="DIFF"/>
     <tableColumn id="5" xr3:uid="{00000000-0010-0000-1900-000005000000}" name="Evidence"/>
     <tableColumn id="3" xr3:uid="{00000000-0010-0000-1900-000003000000}" name="CapabilityID"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleLight2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table26.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="26" xr:uid="{00000000-000C-0000-FFFF-FFFF1C000000}" name="IM_Threats" displayName="IM_Threats" ref="A10:G22" totalsRowShown="0" headerRowDxfId="15" headerRowBorderDxfId="14" tableBorderDxfId="13">
+  <autoFilter ref="A10:G22" xr:uid="{00000000-0009-0000-0100-000021000000}"/>
+  <tableColumns count="7">
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-1C00-000001000000}" name="Scenario" dataDxfId="12"/>
+    <tableColumn id="7" xr3:uid="{00000000-0010-0000-1C00-000007000000}" name="TComm" dataDxfId="11"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-1C00-000002000000}" name="TEF"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-1C00-000003000000}" name="TC"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-1C00-000004000000}" name="LM"/>
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-1C00-000006000000}" name="ScenarioID"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-1C00-000005000000}" name="Capabilities" dataDxfId="10"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleLight2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table27.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="27" xr:uid="{00000000-000C-0000-FFFF-FFFF1B000000}" name="IM_Capabilities" displayName="IM_Capabilities" ref="A2:D7" totalsRowShown="0" headerRowDxfId="19" headerRowBorderDxfId="18" tableBorderDxfId="17">
+  <autoFilter ref="A2:D7" xr:uid="{00000000-0009-0000-0100-000020000000}"/>
+  <tableColumns count="4">
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-1B00-000001000000}" name="Name" dataDxfId="16"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-1B00-000002000000}" name="DIFF"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-1B00-000005000000}" name="Evidence"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-1B00-000003000000}" name="CapabilityID"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleLight2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table28.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="28" xr:uid="{00000000-000C-0000-FFFF-FFFF1E000000}" name="BC_Threats" displayName="BC_Threats" ref="A7:G9" totalsRowShown="0">
+  <autoFilter ref="A7:G9" xr:uid="{00000000-0009-0000-0100-00001D000000}"/>
+  <tableColumns count="7">
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-1E00-000001000000}" name="Scenario" dataDxfId="8"/>
+    <tableColumn id="7" xr3:uid="{00000000-0010-0000-1E00-000007000000}" name="TComm" dataDxfId="7"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-1E00-000002000000}" name="TEF"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-1E00-000003000000}" name="TC"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-1E00-000004000000}" name="LM"/>
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-1E00-000006000000}" name="ScenarioID"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-1E00-000005000000}" name="Capabilities"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleLight2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table29.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="29" xr:uid="{00000000-000C-0000-FFFF-FFFF1D000000}" name="BC_Capabilities" displayName="BC_Capabilities" ref="A2:D4" totalsRowShown="0">
+  <autoFilter ref="A2:D4" xr:uid="{00000000-0009-0000-0100-00001C000000}"/>
+  <tableColumns count="4">
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-1D00-000001000000}" name="Name" dataDxfId="9"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-1D00-000002000000}" name="DIFF"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-1D00-000005000000}" name="Evidence"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-1D00-000003000000}" name="CapabilityID"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1986,65 +3025,7 @@
 </file>
 
 <file path=xl/tables/table30.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="30" xr:uid="{00000000-000C-0000-FFFF-FFFF1C000000}" name="IM_Threats" displayName="IM_Threats" ref="A10:G22" totalsRowShown="0" headerRowDxfId="15" headerRowBorderDxfId="14" tableBorderDxfId="13">
-  <autoFilter ref="A10:G22" xr:uid="{00000000-0009-0000-0100-000021000000}"/>
-  <tableColumns count="7">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-1C00-000001000000}" name="Scenario" dataDxfId="12"/>
-    <tableColumn id="7" xr3:uid="{00000000-0010-0000-1C00-000007000000}" name="TComm" dataDxfId="11"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-1C00-000002000000}" name="TEF"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-1C00-000003000000}" name="TC"/>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-1C00-000004000000}" name="LM"/>
-    <tableColumn id="6" xr3:uid="{00000000-0010-0000-1C00-000006000000}" name="ScenarioID"/>
-    <tableColumn id="5" xr3:uid="{00000000-0010-0000-1C00-000005000000}" name="Capabilities" dataDxfId="10"/>
-  </tableColumns>
-  <tableStyleInfo name="TableStyleLight2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
-</table>
-</file>
-
-<file path=xl/tables/table31.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="31" xr:uid="{00000000-000C-0000-FFFF-FFFF1B000000}" name="IM_Capabilities" displayName="IM_Capabilities" ref="A2:D7" totalsRowShown="0" headerRowDxfId="19" headerRowBorderDxfId="18" tableBorderDxfId="17">
-  <autoFilter ref="A2:D7" xr:uid="{00000000-0009-0000-0100-000020000000}"/>
-  <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-1B00-000001000000}" name="Name" dataDxfId="16"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-1B00-000002000000}" name="DIFF"/>
-    <tableColumn id="5" xr3:uid="{00000000-0010-0000-1B00-000005000000}" name="Evidence"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-1B00-000003000000}" name="CapabilityID"/>
-  </tableColumns>
-  <tableStyleInfo name="TableStyleLight2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
-</table>
-</file>
-
-<file path=xl/tables/table32.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="32" xr:uid="{00000000-000C-0000-FFFF-FFFF1E000000}" name="BC_Threats" displayName="BC_Threats" ref="A7:G9" totalsRowShown="0">
-  <autoFilter ref="A7:G9" xr:uid="{00000000-0009-0000-0100-00001D000000}"/>
-  <tableColumns count="7">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-1E00-000001000000}" name="Scenario" dataDxfId="8"/>
-    <tableColumn id="7" xr3:uid="{00000000-0010-0000-1E00-000007000000}" name="TComm" dataDxfId="7"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-1E00-000002000000}" name="TEF"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-1E00-000003000000}" name="TC"/>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-1E00-000004000000}" name="LM"/>
-    <tableColumn id="6" xr3:uid="{00000000-0010-0000-1E00-000006000000}" name="ScenarioID"/>
-    <tableColumn id="5" xr3:uid="{00000000-0010-0000-1E00-000005000000}" name="Capabilities"/>
-  </tableColumns>
-  <tableStyleInfo name="TableStyleLight2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
-</table>
-</file>
-
-<file path=xl/tables/table33.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="33" xr:uid="{00000000-000C-0000-FFFF-FFFF1D000000}" name="BC_Capabilities" displayName="BC_Capabilities" ref="A2:D4" totalsRowShown="0">
-  <autoFilter ref="A2:D4" xr:uid="{00000000-0009-0000-0100-00001C000000}"/>
-  <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-1D00-000001000000}" name="Name" dataDxfId="9"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-1D00-000002000000}" name="DIFF"/>
-    <tableColumn id="5" xr3:uid="{00000000-0010-0000-1D00-000005000000}" name="Evidence"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-1D00-000003000000}" name="CapabilityID"/>
-  </tableColumns>
-  <tableStyleInfo name="TableStyleLight2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
-</table>
-</file>
-
-<file path=xl/tables/table34.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="34" xr:uid="{00000000-000C-0000-FFFF-FFFF20000000}" name="Privacy_Threats" displayName="Privacy_Threats" ref="A9:G12" totalsRowShown="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="30" xr:uid="{00000000-000C-0000-FFFF-FFFF20000000}" name="Privacy_Threats" displayName="Privacy_Threats" ref="A9:G12" totalsRowShown="0">
   <autoFilter ref="A9:G12" xr:uid="{00000000-0009-0000-0100-000016000000}"/>
   <tableColumns count="7">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-2000-000001000000}" name="Scenario" dataDxfId="2"/>
@@ -2059,8 +3040,8 @@
 </table>
 </file>
 
-<file path=xl/tables/table35.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="35" xr:uid="{00000000-000C-0000-FFFF-FFFF1F000000}" name="Privacy_Capabilities" displayName="Privacy_Capabilities" ref="A2:D6" totalsRowShown="0" headerRowDxfId="6" headerRowBorderDxfId="5" tableBorderDxfId="4">
+<file path=xl/tables/table31.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="31" xr:uid="{00000000-000C-0000-FFFF-FFFF1F000000}" name="Privacy_Capabilities" displayName="Privacy_Capabilities" ref="A2:D6" totalsRowShown="0" headerRowDxfId="6" headerRowBorderDxfId="5" tableBorderDxfId="4">
   <autoFilter ref="A2:D6" xr:uid="{00000000-0009-0000-0100-00000C000000}"/>
   <tableColumns count="4">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-1F00-000001000000}" name="Name" dataDxfId="3"/>
@@ -2073,50 +3054,7 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{00000000-000C-0000-FFFF-FFFF02000000}" name="Table8" displayName="Table8" ref="A11:B13" headerRowCount="0" totalsRowShown="0" tableBorderDxfId="75">
-  <tableColumns count="2">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0200-000001000000}" name="Column1"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0200-000002000000}" name="Column2"/>
-  </tableColumns>
-  <tableStyleInfo name="TableStyleLight2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
-</table>
-</file>
-
-<file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{00000000-000C-0000-FFFF-FFFF01000000}" name="Table7" displayName="Table7" ref="A4:B8" headerRowCount="0" totalsRowShown="0" tableBorderDxfId="76">
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A4:B8">
-    <sortCondition descending="1" ref="A4:A8"/>
-  </sortState>
-  <tableColumns count="2">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0100-000001000000}" name="Column1"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0100-000002000000}" name="Column2"/>
-  </tableColumns>
-  <tableStyleInfo name="TableStyleLight2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
-</table>
-</file>
-
-<file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{00000000-000C-0000-FFFF-FFFF04000000}" name="Table11" displayName="Table11" ref="A21:B23" headerRowCount="0" totalsRowShown="0" tableBorderDxfId="77">
-  <tableColumns count="2">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0400-000001000000}" name="Column1"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0400-000002000000}" name="Column2"/>
-  </tableColumns>
-  <tableStyleInfo name="TableStyleLight2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
-</table>
-</file>
-
-<file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{00000000-000C-0000-FFFF-FFFF03000000}" name="Table9" displayName="Table9" ref="A16:B18" headerRowCount="0" totalsRowShown="0" tableBorderDxfId="74">
-  <tableColumns count="2">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0300-000001000000}" name="Column1"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0300-000002000000}" name="Column2"/>
-  </tableColumns>
-  <tableStyleInfo name="TableStyleLight2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
-</table>
-</file>
-
-<file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{00000000-000C-0000-FFFF-FFFF06000000}" name="ISMP_Threats" displayName="ISMP_Threats" ref="A8:G9" totalsRowShown="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{00000000-000C-0000-FFFF-FFFF06000000}" name="ISMP_Threats" displayName="ISMP_Threats" ref="A8:G9" totalsRowShown="0">
   <autoFilter ref="A8:G9" xr:uid="{00000000-0009-0000-0100-000003000000}"/>
   <tableColumns count="7">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0600-000001000000}" name="Scenario" dataDxfId="79"/>
@@ -2131,14 +3069,72 @@
 </table>
 </file>
 
-<file path=xl/tables/table9.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{00000000-000C-0000-FFFF-FFFF05000000}" name="ISMP_Capabilities" displayName="ISMP_Capabilities" ref="A2:D5" totalsRowShown="0">
+<file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{00000000-000C-0000-FFFF-FFFF05000000}" name="ISMP_Capabilities" displayName="ISMP_Capabilities" ref="A2:D5" totalsRowShown="0">
   <autoFilter ref="A2:D5" xr:uid="{00000000-0009-0000-0100-000002000000}"/>
   <tableColumns count="4">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0500-000001000000}" name="Name" dataDxfId="80"/>
     <tableColumn id="4" xr3:uid="{00000000-0010-0000-0500-000004000000}" name="DIFF"/>
     <tableColumn id="5" xr3:uid="{00000000-0010-0000-0500-000005000000}" name="Evidence"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0500-000002000000}" name="CapabilityID"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleLight2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{00000000-000C-0000-FFFF-FFFF08000000}" name="AC_Threats" displayName="AC_Threats" ref="A7:G9" totalsRowShown="0" headerRowDxfId="69" headerRowBorderDxfId="68" tableBorderDxfId="67">
+  <autoFilter ref="A7:G9" xr:uid="{00000000-0009-0000-0100-00001B000000}"/>
+  <tableColumns count="7">
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0800-000001000000}" name="Scenario" dataDxfId="66"/>
+    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0800-000007000000}" name="TComm" dataDxfId="65"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0800-000002000000}" name="TEF"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0800-000003000000}" name="TC"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0800-000004000000}" name="LM"/>
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0800-000006000000}" name="ScenarioID"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0800-000005000000}" name="Capabilities"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleLight2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{00000000-000C-0000-FFFF-FFFF07000000}" name="AC_Capabilities" displayName="AC_Capabilities" ref="A2:D4" totalsRowShown="0" headerRowDxfId="73" headerRowBorderDxfId="72" tableBorderDxfId="71">
+  <autoFilter ref="A2:D4" xr:uid="{00000000-0009-0000-0100-000004000000}"/>
+  <tableColumns count="4">
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0700-000001000000}" name="Name" dataDxfId="70"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0700-000002000000}" name="DIFF"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0700-000005000000}" name="Evidence"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0700-000003000000}" name="CapabilityID"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleLight2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{00000000-000C-0000-FFFF-FFFF0A000000}" name="HR_Threats" displayName="HR_Threats" ref="A9:G13" totalsRowShown="0">
+  <autoFilter ref="A9:G13" xr:uid="{00000000-0009-0000-0100-000014000000}"/>
+  <tableColumns count="7">
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0A00-000001000000}" name="Scenario" dataDxfId="60"/>
+    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0A00-000007000000}" name="TComm" dataDxfId="59"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0A00-000002000000}" name="TEF"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0A00-000003000000}" name="TC"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0A00-000004000000}" name="LM"/>
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0A00-000006000000}" name="ScenarioID"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0A00-000005000000}" name="Capabilities"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleLight2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table9.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{00000000-000C-0000-FFFF-FFFF09000000}" name="HR_Capabilites" displayName="HR_Capabilites" ref="A2:D6" totalsRowShown="0" headerRowDxfId="64" headerRowBorderDxfId="63" tableBorderDxfId="62">
+  <autoFilter ref="A2:D6" xr:uid="{00000000-0009-0000-0100-00000A000000}"/>
+  <tableColumns count="4">
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0900-000001000000}" name="Name" dataDxfId="61"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0900-000002000000}" name="DIFF"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0900-000005000000}" name="Evidence"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0900-000003000000}" name="CapabilityID"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -2657,10 +3653,10 @@
     </row>
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="7" t="s">
-        <v>116</v>
+        <v>376</v>
       </c>
       <c r="B3" t="s">
-        <v>174</v>
+        <v>347</v>
       </c>
       <c r="C3" t="s">
         <v>43</v>
@@ -2671,10 +3667,10 @@
     </row>
     <row r="4" ht="16" customHeight="1">
       <c r="A4" s="6" t="s">
-        <v>90</v>
+        <v>377</v>
       </c>
       <c r="B4" t="s">
-        <v>172</v>
+        <v>361</v>
       </c>
       <c r="C4" s="12" t="s">
         <v>43</v>
@@ -2718,96 +3714,40 @@
       </c>
     </row>
     <row r="8" ht="32" customHeight="1">
-      <c r="A8" s="6" t="s">
-        <v>180</v>
-      </c>
-      <c r="B8" s="6" t="s">
-        <v>196</v>
-      </c>
-      <c r="C8" t="s">
-        <v>12</v>
-      </c>
-      <c r="D8" t="s">
-        <v>10</v>
-      </c>
-      <c r="E8" t="s">
-        <v>11</v>
-      </c>
-      <c r="F8" t="s">
-        <v>215</v>
-      </c>
-      <c r="G8" t="s">
-        <v>325</v>
-      </c>
+      <c r="A8" s="6"/>
+      <c r="B8" s="6"/>
+      <c r="C8"/>
+      <c r="D8"/>
+      <c r="E8"/>
+      <c r="F8"/>
+      <c r="G8"/>
     </row>
     <row r="9" ht="32" customHeight="1">
-      <c r="A9" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="B9" s="6" t="s">
-        <v>42</v>
-      </c>
-      <c r="C9" t="s">
-        <v>7</v>
-      </c>
-      <c r="D9" t="s">
-        <v>9</v>
-      </c>
-      <c r="E9" t="s">
-        <v>9</v>
-      </c>
-      <c r="F9" t="s">
-        <v>216</v>
-      </c>
-      <c r="G9" t="s">
-        <v>325</v>
-      </c>
+      <c r="A9" s="6"/>
+      <c r="B9" s="6"/>
+      <c r="C9"/>
+      <c r="D9"/>
+      <c r="E9"/>
+      <c r="F9"/>
+      <c r="G9"/>
     </row>
     <row r="10" ht="32" customHeight="1">
-      <c r="A10" s="6" t="s">
-        <v>18</v>
-      </c>
-      <c r="B10" s="6" t="s">
-        <v>195</v>
-      </c>
-      <c r="C10" t="s">
-        <v>7</v>
-      </c>
-      <c r="D10" t="s">
-        <v>11</v>
-      </c>
-      <c r="E10" t="s">
-        <v>9</v>
-      </c>
-      <c r="F10" t="s">
-        <v>217</v>
-      </c>
-      <c r="G10" t="s">
-        <v>325</v>
-      </c>
+      <c r="A10" s="6"/>
+      <c r="B10" s="6"/>
+      <c r="C10"/>
+      <c r="D10"/>
+      <c r="E10"/>
+      <c r="F10"/>
+      <c r="G10"/>
     </row>
     <row r="11" ht="32" customHeight="1">
-      <c r="A11" s="6" t="s">
-        <v>17</v>
-      </c>
-      <c r="B11" s="6" t="s">
-        <v>195</v>
-      </c>
-      <c r="C11" t="s">
-        <v>8</v>
-      </c>
-      <c r="D11" t="s">
-        <v>9</v>
-      </c>
-      <c r="E11" t="s">
-        <v>9</v>
-      </c>
-      <c r="F11" t="s">
-        <v>218</v>
-      </c>
-      <c r="G11" t="s">
-        <v>325</v>
-      </c>
+      <c r="A11" s="6"/>
+      <c r="B11" s="6"/>
+      <c r="C11"/>
+      <c r="D11"/>
+      <c r="E11"/>
+      <c r="F11"/>
+      <c r="G11"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -2831,8 +3771,8 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="5" orientation="landscape"/>
   <tableParts count="2">
-    <tablePart r:id="rId20"/>
-    <tablePart r:id="rId21"/>
+    <tablePart r:id="rId16"/>
+    <tablePart r:id="rId17"/>
   </tableParts>
 </worksheet>
 </file>
@@ -2874,10 +3814,10 @@
     </row>
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="6" t="s">
-        <v>94</v>
+        <v>378</v>
       </c>
       <c r="B3" t="s">
-        <v>175</v>
+        <v>356</v>
       </c>
       <c r="C3" t="s">
         <v>43</v>
@@ -2888,10 +3828,10 @@
     </row>
     <row r="4" ht="16" customHeight="1">
       <c r="A4" s="6" t="s">
-        <v>112</v>
+        <v>379</v>
       </c>
       <c r="B4" t="s">
-        <v>175</v>
+        <v>356</v>
       </c>
       <c r="C4" t="s">
         <v>43</v>
@@ -2938,73 +3878,31 @@
       </c>
     </row>
     <row r="8" ht="32" customHeight="1">
-      <c r="A8" s="6" t="s">
-        <v>39</v>
-      </c>
-      <c r="B8" s="6" t="s">
-        <v>42</v>
-      </c>
-      <c r="C8" t="s">
-        <v>12</v>
-      </c>
-      <c r="D8" t="s">
-        <v>9</v>
-      </c>
-      <c r="E8" t="s">
-        <v>10</v>
-      </c>
-      <c r="F8" t="s">
-        <v>219</v>
-      </c>
-      <c r="G8" t="s">
-        <v>285</v>
-      </c>
+      <c r="A8" s="6"/>
+      <c r="B8" s="6"/>
+      <c r="C8"/>
+      <c r="D8"/>
+      <c r="E8"/>
+      <c r="F8"/>
+      <c r="G8"/>
     </row>
     <row r="9" ht="32" customHeight="1">
-      <c r="A9" s="6" t="s">
-        <v>95</v>
-      </c>
-      <c r="B9" s="6" t="s">
-        <v>42</v>
-      </c>
-      <c r="C9" t="s">
-        <v>8</v>
-      </c>
-      <c r="D9" t="s">
-        <v>10</v>
-      </c>
-      <c r="E9" t="s">
-        <v>10</v>
-      </c>
-      <c r="F9" t="s">
-        <v>220</v>
-      </c>
-      <c r="G9" t="s">
-        <v>285</v>
-      </c>
+      <c r="A9" s="6"/>
+      <c r="B9" s="6"/>
+      <c r="C9"/>
+      <c r="D9"/>
+      <c r="E9"/>
+      <c r="F9"/>
+      <c r="G9"/>
     </row>
     <row r="10" ht="32" customHeight="1">
-      <c r="A10" s="6" t="s">
-        <v>181</v>
-      </c>
-      <c r="B10" s="6" t="s">
-        <v>42</v>
-      </c>
-      <c r="C10" t="s">
-        <v>8</v>
-      </c>
-      <c r="D10" t="s">
-        <v>9</v>
-      </c>
-      <c r="E10" t="s">
-        <v>9</v>
-      </c>
-      <c r="F10" t="s">
-        <v>221</v>
-      </c>
-      <c r="G10" t="s">
-        <v>285</v>
-      </c>
+      <c r="A10" s="6"/>
+      <c r="B10" s="6"/>
+      <c r="C10"/>
+      <c r="D10"/>
+      <c r="E10"/>
+      <c r="F10"/>
+      <c r="G10"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -3028,8 +3926,8 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="5" orientation="landscape"/>
   <tableParts count="2">
-    <tablePart r:id="rId22"/>
-    <tablePart r:id="rId23"/>
+    <tablePart r:id="rId18"/>
+    <tablePart r:id="rId19"/>
   </tableParts>
 </worksheet>
 </file>
@@ -3071,10 +3969,10 @@
     </row>
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="6" t="s">
-        <v>96</v>
+        <v>380</v>
       </c>
       <c r="B3" t="s">
-        <v>173</v>
+        <v>350</v>
       </c>
       <c r="C3" t="s">
         <v>43</v>
@@ -3085,10 +3983,10 @@
     </row>
     <row r="4" ht="32" customHeight="1">
       <c r="A4" s="6" t="s">
-        <v>118</v>
+        <v>381</v>
       </c>
       <c r="B4" t="s">
-        <v>173</v>
+        <v>350</v>
       </c>
       <c r="C4" t="s">
         <v>43</v>
@@ -3099,10 +3997,10 @@
     </row>
     <row r="5" ht="32" customHeight="1">
       <c r="A5" s="6" t="s">
-        <v>97</v>
+        <v>382</v>
       </c>
       <c r="B5" t="s">
-        <v>172</v>
+        <v>361</v>
       </c>
       <c r="C5" t="s">
         <v>43</v>
@@ -3113,10 +4011,10 @@
     </row>
     <row r="6" ht="16" customHeight="1">
       <c r="A6" s="6" t="s">
-        <v>98</v>
+        <v>383</v>
       </c>
       <c r="B6" t="s">
-        <v>175</v>
+        <v>356</v>
       </c>
       <c r="C6" t="s">
         <v>43</v>
@@ -3160,96 +4058,40 @@
       </c>
     </row>
     <row r="10" ht="32" customHeight="1">
-      <c r="A10" s="6" t="s">
-        <v>146</v>
-      </c>
-      <c r="B10" s="6" t="s">
-        <v>197</v>
-      </c>
-      <c r="C10" t="s">
-        <v>8</v>
-      </c>
-      <c r="D10" t="s">
-        <v>9</v>
-      </c>
-      <c r="E10" t="s">
-        <v>9</v>
-      </c>
-      <c r="F10" t="s">
-        <v>222</v>
-      </c>
-      <c r="G10" t="s">
-        <v>290</v>
-      </c>
+      <c r="A10" s="6"/>
+      <c r="B10" s="6"/>
+      <c r="C10"/>
+      <c r="D10"/>
+      <c r="E10"/>
+      <c r="F10"/>
+      <c r="G10"/>
     </row>
     <row r="11" ht="16" customHeight="1">
-      <c r="A11" s="6" t="s">
-        <v>37</v>
-      </c>
-      <c r="B11" s="6" t="s">
-        <v>198</v>
-      </c>
-      <c r="C11" t="s">
-        <v>8</v>
-      </c>
-      <c r="D11" t="s">
-        <v>11</v>
-      </c>
-      <c r="E11" t="s">
-        <v>11</v>
-      </c>
-      <c r="F11" t="s">
-        <v>223</v>
-      </c>
-      <c r="G11" t="s">
-        <v>290</v>
-      </c>
+      <c r="A11" s="6"/>
+      <c r="B11" s="6"/>
+      <c r="C11"/>
+      <c r="D11"/>
+      <c r="E11"/>
+      <c r="F11"/>
+      <c r="G11"/>
     </row>
     <row r="12" ht="32" customHeight="1">
-      <c r="A12" s="6" t="s">
-        <v>38</v>
-      </c>
-      <c r="B12" s="6" t="s">
-        <v>42</v>
-      </c>
-      <c r="C12" t="s">
-        <v>8</v>
-      </c>
-      <c r="D12" t="s">
-        <v>11</v>
-      </c>
-      <c r="E12" t="s">
-        <v>9</v>
-      </c>
-      <c r="F12" t="s">
-        <v>224</v>
-      </c>
-      <c r="G12" t="s">
-        <v>290</v>
-      </c>
+      <c r="A12" s="6"/>
+      <c r="B12" s="6"/>
+      <c r="C12"/>
+      <c r="D12"/>
+      <c r="E12"/>
+      <c r="F12"/>
+      <c r="G12"/>
     </row>
     <row r="13" ht="16" customHeight="1">
-      <c r="A13" s="6" t="s">
-        <v>36</v>
-      </c>
-      <c r="B13" s="6" t="s">
-        <v>197</v>
-      </c>
-      <c r="C13" t="s">
-        <v>12</v>
-      </c>
-      <c r="D13" t="s">
-        <v>10</v>
-      </c>
-      <c r="E13" t="s">
-        <v>9</v>
-      </c>
-      <c r="F13" t="s">
-        <v>225</v>
-      </c>
-      <c r="G13" t="s">
-        <v>290</v>
-      </c>
+      <c r="A13" s="6"/>
+      <c r="B13" s="6"/>
+      <c r="C13"/>
+      <c r="D13"/>
+      <c r="E13"/>
+      <c r="F13"/>
+      <c r="G13"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -3273,8 +4115,8 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="5" orientation="landscape"/>
   <tableParts count="2">
-    <tablePart r:id="rId24"/>
-    <tablePart r:id="rId25"/>
+    <tablePart r:id="rId20"/>
+    <tablePart r:id="rId21"/>
   </tableParts>
 </worksheet>
 </file>
@@ -3316,10 +4158,10 @@
     </row>
     <row r="3" ht="16" customHeight="1">
       <c r="A3" s="6" t="s">
-        <v>110</v>
+        <v>384</v>
       </c>
       <c r="B3" t="s">
-        <v>173</v>
+        <v>350</v>
       </c>
       <c r="C3" t="s">
         <v>43</v>
@@ -3330,10 +4172,10 @@
     </row>
     <row r="4" ht="16" customHeight="1">
       <c r="A4" s="6" t="s">
-        <v>123</v>
+        <v>385</v>
       </c>
       <c r="B4" t="s">
-        <v>175</v>
+        <v>356</v>
       </c>
       <c r="C4" t="s">
         <v>43</v>
@@ -3344,10 +4186,10 @@
     </row>
     <row r="5" ht="32" customHeight="1">
       <c r="A5" s="6" t="s">
-        <v>122</v>
+        <v>386</v>
       </c>
       <c r="B5" t="s">
-        <v>174</v>
+        <v>347</v>
       </c>
       <c r="C5" t="s">
         <v>43</v>
@@ -3358,10 +4200,10 @@
     </row>
     <row r="6" ht="32" customHeight="1">
       <c r="A6" s="6" t="s">
-        <v>121</v>
+        <v>387</v>
       </c>
       <c r="B6" t="s">
-        <v>175</v>
+        <v>356</v>
       </c>
       <c r="C6" t="s">
         <v>43</v>
@@ -3372,10 +4214,10 @@
     </row>
     <row r="7" ht="16" customHeight="1">
       <c r="A7" s="6" t="s">
-        <v>124</v>
+        <v>388</v>
       </c>
       <c r="B7" t="s">
-        <v>174</v>
+        <v>347</v>
       </c>
       <c r="C7" t="s">
         <v>43</v>
@@ -3386,10 +4228,10 @@
     </row>
     <row r="8" ht="16" customHeight="1">
       <c r="A8" s="6" t="s">
-        <v>125</v>
+        <v>389</v>
       </c>
       <c r="B8" t="s">
-        <v>174</v>
+        <v>347</v>
       </c>
       <c r="C8" t="s">
         <v>43</v>
@@ -3400,10 +4242,10 @@
     </row>
     <row r="9" ht="32" customHeight="1">
       <c r="A9" s="6" t="s">
-        <v>126</v>
+        <v>390</v>
       </c>
       <c r="B9" t="s">
-        <v>171</v>
+        <v>370</v>
       </c>
       <c r="C9" t="s">
         <v>43</v>
@@ -3414,10 +4256,10 @@
     </row>
     <row r="10" ht="32" customHeight="1">
       <c r="A10" s="6" t="s">
-        <v>127</v>
+        <v>391</v>
       </c>
       <c r="B10" t="s">
-        <v>172</v>
+        <v>361</v>
       </c>
       <c r="C10" t="s">
         <v>43</v>
@@ -3428,10 +4270,10 @@
     </row>
     <row r="11" ht="32" customHeight="1">
       <c r="A11" s="6" t="s">
-        <v>128</v>
+        <v>392</v>
       </c>
       <c r="B11" t="s">
-        <v>173</v>
+        <v>350</v>
       </c>
       <c r="C11" t="s">
         <v>43</v>
@@ -3442,10 +4284,10 @@
     </row>
     <row r="12" ht="16" customHeight="1">
       <c r="A12" s="6" t="s">
-        <v>107</v>
+        <v>393</v>
       </c>
       <c r="B12" t="s">
-        <v>172</v>
+        <v>361</v>
       </c>
       <c r="C12" t="s">
         <v>43</v>
@@ -3456,10 +4298,10 @@
     </row>
     <row r="13" ht="32" customHeight="1">
       <c r="A13" s="6" t="s">
-        <v>185</v>
+        <v>394</v>
       </c>
       <c r="B13" t="s">
-        <v>173</v>
+        <v>350</v>
       </c>
       <c r="C13" t="s">
         <v>43</v>
@@ -3470,10 +4312,10 @@
     </row>
     <row r="14" ht="16" customHeight="1">
       <c r="A14" s="6" t="s">
-        <v>131</v>
+        <v>395</v>
       </c>
       <c r="B14" t="s">
-        <v>175</v>
+        <v>356</v>
       </c>
       <c r="C14" t="s">
         <v>43</v>
@@ -3484,10 +4326,10 @@
     </row>
     <row r="15" ht="16" customHeight="1">
       <c r="A15" s="6" t="s">
-        <v>130</v>
+        <v>396</v>
       </c>
       <c r="B15" t="s">
-        <v>175</v>
+        <v>356</v>
       </c>
       <c r="C15" t="s">
         <v>43</v>
@@ -3498,10 +4340,10 @@
     </row>
     <row r="16" ht="16" customHeight="1">
       <c r="A16" s="6" t="s">
-        <v>129</v>
+        <v>397</v>
       </c>
       <c r="B16" t="s">
-        <v>175</v>
+        <v>356</v>
       </c>
       <c r="C16" t="s">
         <v>43</v>
@@ -3548,188 +4390,76 @@
       </c>
     </row>
     <row r="20" ht="80" customHeight="1">
-      <c r="A20" s="6" t="s">
-        <v>186</v>
-      </c>
-      <c r="B20" t="s">
-        <v>42</v>
-      </c>
-      <c r="C20" t="s">
-        <v>7</v>
-      </c>
-      <c r="D20" t="s">
-        <v>10</v>
-      </c>
-      <c r="E20" t="s">
-        <v>9</v>
-      </c>
-      <c r="F20" t="s">
-        <v>226</v>
-      </c>
-      <c r="G20" s="6" t="s">
-        <v>305</v>
-      </c>
+      <c r="A20" s="6"/>
+      <c r="B20"/>
+      <c r="C20"/>
+      <c r="D20"/>
+      <c r="E20"/>
+      <c r="F20"/>
+      <c r="G20" s="6"/>
     </row>
     <row r="21" ht="80" customHeight="1">
-      <c r="A21" s="6" t="s">
-        <v>32</v>
-      </c>
-      <c r="B21" t="s">
-        <v>42</v>
-      </c>
-      <c r="C21" t="s">
-        <v>8</v>
-      </c>
-      <c r="D21" t="s">
-        <v>11</v>
-      </c>
-      <c r="E21" t="s">
-        <v>10</v>
-      </c>
-      <c r="F21" t="s">
-        <v>227</v>
-      </c>
-      <c r="G21" s="6" t="s">
-        <v>305</v>
-      </c>
+      <c r="A21" s="6"/>
+      <c r="B21"/>
+      <c r="C21"/>
+      <c r="D21"/>
+      <c r="E21"/>
+      <c r="F21"/>
+      <c r="G21" s="6"/>
     </row>
     <row r="22" ht="80" customHeight="1">
-      <c r="A22" s="6" t="s">
-        <v>34</v>
-      </c>
-      <c r="B22" t="s">
-        <v>195</v>
-      </c>
-      <c r="C22" t="s">
-        <v>8</v>
-      </c>
-      <c r="D22" t="s">
-        <v>11</v>
-      </c>
-      <c r="E22" t="s">
-        <v>9</v>
-      </c>
-      <c r="F22" t="s">
-        <v>228</v>
-      </c>
-      <c r="G22" s="6" t="s">
-        <v>305</v>
-      </c>
+      <c r="A22" s="6"/>
+      <c r="B22"/>
+      <c r="C22"/>
+      <c r="D22"/>
+      <c r="E22"/>
+      <c r="F22"/>
+      <c r="G22" s="6"/>
     </row>
     <row r="23" ht="80" customHeight="1">
-      <c r="A23" s="6" t="s">
-        <v>35</v>
-      </c>
-      <c r="B23" t="s">
-        <v>195</v>
-      </c>
-      <c r="C23" t="s">
-        <v>8</v>
-      </c>
-      <c r="D23" t="s">
-        <v>9</v>
-      </c>
-      <c r="E23" t="s">
-        <v>10</v>
-      </c>
-      <c r="F23" t="s">
-        <v>229</v>
-      </c>
-      <c r="G23" s="6" t="s">
-        <v>305</v>
-      </c>
+      <c r="A23" s="6"/>
+      <c r="B23"/>
+      <c r="C23"/>
+      <c r="D23"/>
+      <c r="E23"/>
+      <c r="F23"/>
+      <c r="G23" s="6"/>
     </row>
     <row r="24" ht="80" customHeight="1">
-      <c r="A24" s="6" t="s">
-        <v>33</v>
-      </c>
-      <c r="B24" t="s">
-        <v>193</v>
-      </c>
-      <c r="C24" t="s">
-        <v>12</v>
-      </c>
-      <c r="D24" t="s">
-        <v>10</v>
-      </c>
-      <c r="E24" t="s">
-        <v>10</v>
-      </c>
-      <c r="F24" t="s">
-        <v>230</v>
-      </c>
-      <c r="G24" s="6" t="s">
-        <v>305</v>
-      </c>
+      <c r="A24" s="6"/>
+      <c r="B24"/>
+      <c r="C24"/>
+      <c r="D24"/>
+      <c r="E24"/>
+      <c r="F24"/>
+      <c r="G24" s="6"/>
     </row>
     <row r="25" ht="16" customHeight="1">
-      <c r="A25" s="6" t="s">
-        <v>140</v>
-      </c>
-      <c r="B25" t="s">
-        <v>195</v>
-      </c>
-      <c r="C25" t="s">
-        <v>7</v>
-      </c>
-      <c r="D25" t="s">
-        <v>11</v>
-      </c>
-      <c r="E25" t="s">
-        <v>10</v>
-      </c>
-      <c r="F25" t="s">
-        <v>231</v>
-      </c>
-      <c r="G25" s="6" t="s">
-        <v>306</v>
-      </c>
+      <c r="A25" s="6"/>
+      <c r="B25"/>
+      <c r="C25"/>
+      <c r="D25"/>
+      <c r="E25"/>
+      <c r="F25"/>
+      <c r="G25" s="6"/>
     </row>
     <row r="26" ht="16" customHeight="1">
-      <c r="A26" s="6" t="s">
-        <v>141</v>
-      </c>
-      <c r="B26" t="s">
-        <v>195</v>
-      </c>
-      <c r="C26" t="s">
-        <v>12</v>
-      </c>
-      <c r="D26" t="s">
-        <v>9</v>
-      </c>
-      <c r="E26" t="s">
-        <v>10</v>
-      </c>
-      <c r="F26" t="s">
-        <v>232</v>
-      </c>
-      <c r="G26" s="6" t="s">
-        <v>306</v>
-      </c>
+      <c r="A26" s="6"/>
+      <c r="B26"/>
+      <c r="C26"/>
+      <c r="D26"/>
+      <c r="E26"/>
+      <c r="F26"/>
+      <c r="G26" s="6"/>
     </row>
     <row r="27" ht="32" customHeight="1">
-      <c r="A27" s="6" t="s">
-        <v>176</v>
-      </c>
-      <c r="B27" s="6" t="s">
-        <v>196</v>
-      </c>
-      <c r="C27" t="s">
-        <v>12</v>
-      </c>
-      <c r="D27" t="s">
-        <v>10</v>
-      </c>
-      <c r="E27" t="s">
-        <v>9</v>
-      </c>
-      <c r="F27" t="s">
-        <v>233</v>
-      </c>
-      <c r="G27" s="6" t="s">
-        <v>306</v>
-      </c>
+      <c r="A27" s="6"/>
+      <c r="B27" s="6"/>
+      <c r="C27"/>
+      <c r="D27"/>
+      <c r="E27"/>
+      <c r="F27"/>
+      <c r="G27" s="6"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -3753,8 +4483,8 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
   <tableParts count="2">
-    <tablePart r:id="rId26"/>
-    <tablePart r:id="rId27"/>
+    <tablePart r:id="rId22"/>
+    <tablePart r:id="rId23"/>
   </tableParts>
 </worksheet>
 </file>
@@ -3795,10 +4525,10 @@
     </row>
     <row r="3" ht="16" customHeight="1">
       <c r="A3" s="6" t="s">
-        <v>111</v>
+        <v>398</v>
       </c>
       <c r="B3" t="s">
-        <v>173</v>
+        <v>350</v>
       </c>
       <c r="C3" t="s">
         <v>43</v>
@@ -3809,10 +4539,10 @@
     </row>
     <row r="4" ht="32" customHeight="1">
       <c r="A4" s="6" t="s">
-        <v>113</v>
+        <v>399</v>
       </c>
       <c r="B4" t="s">
-        <v>172</v>
+        <v>361</v>
       </c>
       <c r="C4" t="s">
         <v>43</v>
@@ -3856,27 +4586,13 @@
       </c>
     </row>
     <row r="8" ht="32" customHeight="1">
-      <c r="A8" s="6" t="s">
-        <v>32</v>
-      </c>
-      <c r="B8" s="6" t="s">
-        <v>42</v>
-      </c>
-      <c r="C8" t="s">
-        <v>8</v>
-      </c>
-      <c r="D8" t="s">
-        <v>11</v>
-      </c>
-      <c r="E8" t="s">
-        <v>9</v>
-      </c>
-      <c r="F8" t="s">
-        <v>234</v>
-      </c>
-      <c r="G8" t="s">
-        <v>309</v>
-      </c>
+      <c r="A8" s="6"/>
+      <c r="B8" s="6"/>
+      <c r="C8"/>
+      <c r="D8"/>
+      <c r="E8"/>
+      <c r="F8"/>
+      <c r="G8"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -3900,8 +4616,8 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="5" orientation="landscape"/>
   <tableParts count="2">
-    <tablePart r:id="rId28"/>
-    <tablePart r:id="rId29"/>
+    <tablePart r:id="rId24"/>
+    <tablePart r:id="rId25"/>
   </tableParts>
 </worksheet>
 </file>
@@ -3943,10 +4659,10 @@
     </row>
     <row r="3" ht="16" customHeight="1">
       <c r="A3" s="6" t="s">
-        <v>134</v>
+        <v>400</v>
       </c>
       <c r="B3" t="s">
-        <v>175</v>
+        <v>356</v>
       </c>
       <c r="C3" t="s">
         <v>43</v>
@@ -3957,10 +4673,10 @@
     </row>
     <row r="4" ht="32" customHeight="1">
       <c r="A4" s="6" t="s">
-        <v>183</v>
+        <v>401</v>
       </c>
       <c r="B4" t="s">
-        <v>175</v>
+        <v>356</v>
       </c>
       <c r="C4" t="s">
         <v>43</v>
@@ -3971,10 +4687,10 @@
     </row>
     <row r="5" ht="16" customHeight="1">
       <c r="A5" s="6" t="s">
-        <v>135</v>
+        <v>402</v>
       </c>
       <c r="B5" t="s">
-        <v>171</v>
+        <v>370</v>
       </c>
       <c r="C5" t="s">
         <v>43</v>
@@ -3985,10 +4701,10 @@
     </row>
     <row r="6" ht="16" customHeight="1">
       <c r="A6" s="6" t="s">
-        <v>136</v>
+        <v>403</v>
       </c>
       <c r="B6" t="s">
-        <v>171</v>
+        <v>370</v>
       </c>
       <c r="C6" t="s">
         <v>43</v>
@@ -3999,10 +4715,10 @@
     </row>
     <row r="7" ht="16" customHeight="1">
       <c r="A7" s="6" t="s">
-        <v>137</v>
+        <v>404</v>
       </c>
       <c r="B7" t="s">
-        <v>172</v>
+        <v>361</v>
       </c>
       <c r="C7" t="s">
         <v>43</v>
@@ -4046,280 +4762,112 @@
       </c>
     </row>
     <row r="11" ht="48" customHeight="1">
-      <c r="A11" s="6" t="s">
-        <v>41</v>
-      </c>
-      <c r="B11" s="6" t="s">
-        <v>42</v>
-      </c>
-      <c r="C11" t="s">
-        <v>12</v>
-      </c>
-      <c r="D11" t="s">
-        <v>11</v>
-      </c>
-      <c r="E11" t="s">
-        <v>10</v>
-      </c>
-      <c r="F11" t="s">
-        <v>235</v>
-      </c>
-      <c r="G11" s="6" t="s">
-        <v>315</v>
-      </c>
+      <c r="A11" s="6"/>
+      <c r="B11" s="6"/>
+      <c r="C11"/>
+      <c r="D11"/>
+      <c r="E11"/>
+      <c r="F11"/>
+      <c r="G11" s="6"/>
     </row>
     <row r="12" ht="48" customHeight="1">
-      <c r="A12" s="6" t="s">
-        <v>184</v>
-      </c>
-      <c r="B12" s="6" t="s">
-        <v>42</v>
-      </c>
-      <c r="C12" t="s">
-        <v>8</v>
-      </c>
-      <c r="D12" t="s">
-        <v>11</v>
-      </c>
-      <c r="E12" t="s">
-        <v>9</v>
-      </c>
-      <c r="F12" t="s">
-        <v>236</v>
-      </c>
-      <c r="G12" s="6" t="s">
-        <v>315</v>
-      </c>
+      <c r="A12" s="6"/>
+      <c r="B12" s="6"/>
+      <c r="C12"/>
+      <c r="D12"/>
+      <c r="E12"/>
+      <c r="F12"/>
+      <c r="G12" s="6"/>
     </row>
     <row r="13" ht="48" customHeight="1">
-      <c r="A13" s="6" t="s">
-        <v>25</v>
-      </c>
-      <c r="B13" s="6" t="s">
-        <v>42</v>
-      </c>
-      <c r="C13" t="s">
-        <v>12</v>
-      </c>
-      <c r="D13" t="s">
-        <v>9</v>
-      </c>
-      <c r="E13" t="s">
-        <v>9</v>
-      </c>
-      <c r="F13" t="s">
-        <v>237</v>
-      </c>
-      <c r="G13" s="6" t="s">
-        <v>315</v>
-      </c>
+      <c r="A13" s="6"/>
+      <c r="B13" s="6"/>
+      <c r="C13"/>
+      <c r="D13"/>
+      <c r="E13"/>
+      <c r="F13"/>
+      <c r="G13" s="6"/>
     </row>
     <row r="14" ht="48" customHeight="1">
-      <c r="A14" s="6" t="s">
-        <v>182</v>
-      </c>
-      <c r="B14" s="6" t="s">
-        <v>195</v>
-      </c>
-      <c r="C14" t="s">
-        <v>7</v>
-      </c>
-      <c r="D14" t="s">
-        <v>9</v>
-      </c>
-      <c r="E14" t="s">
-        <v>9</v>
-      </c>
-      <c r="F14" t="s">
-        <v>238</v>
-      </c>
-      <c r="G14" s="6" t="s">
-        <v>315</v>
-      </c>
+      <c r="A14" s="6"/>
+      <c r="B14" s="6"/>
+      <c r="C14"/>
+      <c r="D14"/>
+      <c r="E14"/>
+      <c r="F14"/>
+      <c r="G14" s="6"/>
     </row>
     <row r="15" ht="48" customHeight="1">
-      <c r="A15" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="B15" s="6" t="s">
-        <v>195</v>
-      </c>
-      <c r="C15" t="s">
-        <v>12</v>
-      </c>
-      <c r="D15" t="s">
-        <v>10</v>
-      </c>
-      <c r="E15" t="s">
-        <v>9</v>
-      </c>
-      <c r="F15" t="s">
-        <v>239</v>
-      </c>
-      <c r="G15" s="6" t="s">
-        <v>315</v>
-      </c>
+      <c r="A15" s="6"/>
+      <c r="B15" s="6"/>
+      <c r="C15"/>
+      <c r="D15"/>
+      <c r="E15"/>
+      <c r="F15"/>
+      <c r="G15" s="6"/>
     </row>
     <row r="16" ht="48" customHeight="1">
-      <c r="A16" s="6" t="s">
-        <v>27</v>
-      </c>
-      <c r="B16" s="6" t="s">
-        <v>195</v>
-      </c>
-      <c r="C16" t="s">
-        <v>7</v>
-      </c>
-      <c r="D16" t="s">
-        <v>11</v>
-      </c>
-      <c r="E16" t="s">
-        <v>9</v>
-      </c>
-      <c r="F16" t="s">
-        <v>240</v>
-      </c>
-      <c r="G16" s="6" t="s">
-        <v>315</v>
-      </c>
+      <c r="A16" s="6"/>
+      <c r="B16" s="6"/>
+      <c r="C16"/>
+      <c r="D16"/>
+      <c r="E16"/>
+      <c r="F16"/>
+      <c r="G16" s="6"/>
     </row>
     <row r="17" ht="16" customHeight="1">
-      <c r="A17" s="6" t="s">
-        <v>28</v>
-      </c>
-      <c r="B17" s="6" t="s">
-        <v>199</v>
-      </c>
-      <c r="C17" t="s">
-        <v>8</v>
-      </c>
-      <c r="D17" t="s">
-        <v>10</v>
-      </c>
-      <c r="E17" t="s">
-        <v>9</v>
-      </c>
-      <c r="F17" t="s">
-        <v>241</v>
-      </c>
-      <c r="G17" s="6" t="s">
-        <v>314</v>
-      </c>
+      <c r="A17" s="6"/>
+      <c r="B17" s="6"/>
+      <c r="C17"/>
+      <c r="D17"/>
+      <c r="E17"/>
+      <c r="F17"/>
+      <c r="G17" s="6"/>
     </row>
     <row r="18" ht="32" customHeight="1">
-      <c r="A18" s="6" t="s">
-        <v>29</v>
-      </c>
-      <c r="B18" s="6" t="s">
-        <v>42</v>
-      </c>
-      <c r="C18" t="s">
-        <v>12</v>
-      </c>
-      <c r="D18" t="s">
-        <v>9</v>
-      </c>
-      <c r="E18" t="s">
-        <v>10</v>
-      </c>
-      <c r="F18" t="s">
-        <v>242</v>
-      </c>
-      <c r="G18" s="6" t="s">
-        <v>314</v>
-      </c>
+      <c r="A18" s="6"/>
+      <c r="B18" s="6"/>
+      <c r="C18"/>
+      <c r="D18"/>
+      <c r="E18"/>
+      <c r="F18"/>
+      <c r="G18" s="6"/>
     </row>
     <row r="19" ht="48" customHeight="1">
-      <c r="A19" s="6" t="s">
-        <v>142</v>
-      </c>
-      <c r="B19" s="6" t="s">
-        <v>195</v>
-      </c>
-      <c r="C19" t="s">
-        <v>8</v>
-      </c>
-      <c r="D19" t="s">
-        <v>11</v>
-      </c>
-      <c r="E19" t="s">
-        <v>9</v>
-      </c>
-      <c r="F19" t="s">
-        <v>243</v>
-      </c>
-      <c r="G19" s="6" t="s">
-        <v>315</v>
-      </c>
+      <c r="A19" s="6"/>
+      <c r="B19" s="6"/>
+      <c r="C19"/>
+      <c r="D19"/>
+      <c r="E19"/>
+      <c r="F19"/>
+      <c r="G19" s="6"/>
     </row>
     <row r="20" ht="48" customHeight="1">
-      <c r="A20" s="6" t="s">
-        <v>143</v>
-      </c>
-      <c r="B20" s="6" t="s">
-        <v>195</v>
-      </c>
-      <c r="C20" t="s">
-        <v>8</v>
-      </c>
-      <c r="D20" t="s">
-        <v>11</v>
-      </c>
-      <c r="E20" t="s">
-        <v>9</v>
-      </c>
-      <c r="F20" t="s">
-        <v>244</v>
-      </c>
-      <c r="G20" s="6" t="s">
-        <v>315</v>
-      </c>
+      <c r="A20" s="6"/>
+      <c r="B20" s="6"/>
+      <c r="C20"/>
+      <c r="D20"/>
+      <c r="E20"/>
+      <c r="F20"/>
+      <c r="G20" s="6"/>
     </row>
     <row r="21" ht="48" customHeight="1">
-      <c r="A21" s="6" t="s">
-        <v>144</v>
-      </c>
-      <c r="B21" s="6" t="s">
-        <v>195</v>
-      </c>
-      <c r="C21" t="s">
-        <v>7</v>
-      </c>
-      <c r="D21" t="s">
-        <v>9</v>
-      </c>
-      <c r="E21" t="s">
-        <v>10</v>
-      </c>
-      <c r="F21" t="s">
-        <v>245</v>
-      </c>
-      <c r="G21" s="6" t="s">
-        <v>315</v>
-      </c>
+      <c r="A21" s="6"/>
+      <c r="B21" s="6"/>
+      <c r="C21"/>
+      <c r="D21"/>
+      <c r="E21"/>
+      <c r="F21"/>
+      <c r="G21" s="6"/>
     </row>
     <row r="22" ht="48" customHeight="1">
-      <c r="A22" s="6" t="s">
-        <v>145</v>
-      </c>
-      <c r="B22" s="6" t="s">
-        <v>42</v>
-      </c>
-      <c r="C22" t="s">
-        <v>12</v>
-      </c>
-      <c r="D22" t="s">
-        <v>9</v>
-      </c>
-      <c r="E22" t="s">
-        <v>9</v>
-      </c>
-      <c r="F22" t="s">
-        <v>246</v>
-      </c>
-      <c r="G22" s="6" t="s">
-        <v>315</v>
-      </c>
+      <c r="A22" s="6"/>
+      <c r="B22" s="6"/>
+      <c r="C22"/>
+      <c r="D22"/>
+      <c r="E22"/>
+      <c r="F22"/>
+      <c r="G22" s="6"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -4343,8 +4891,8 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="landscape"/>
   <tableParts count="2">
-    <tablePart r:id="rId30"/>
-    <tablePart r:id="rId31"/>
+    <tablePart r:id="rId26"/>
+    <tablePart r:id="rId27"/>
   </tableParts>
 </worksheet>
 </file>
@@ -4385,10 +4933,10 @@
     </row>
     <row r="3" ht="16" customHeight="1">
       <c r="A3" s="6" t="s">
-        <v>108</v>
+        <v>405</v>
       </c>
       <c r="B3" t="s">
-        <v>172</v>
+        <v>361</v>
       </c>
       <c r="C3" t="s">
         <v>43</v>
@@ -4399,10 +4947,10 @@
     </row>
     <row r="4" ht="32" customHeight="1">
       <c r="A4" s="6" t="s">
-        <v>109</v>
+        <v>406</v>
       </c>
       <c r="B4" t="s">
-        <v>173</v>
+        <v>350</v>
       </c>
       <c r="C4" t="s">
         <v>43</v>
@@ -4446,50 +4994,22 @@
       </c>
     </row>
     <row r="8" ht="16" customHeight="1">
-      <c r="A8" s="6" t="s">
-        <v>147</v>
-      </c>
-      <c r="B8" s="6" t="s">
-        <v>198</v>
-      </c>
-      <c r="C8" t="s">
-        <v>8</v>
-      </c>
-      <c r="D8" t="s">
-        <v>11</v>
-      </c>
-      <c r="E8" t="s">
-        <v>11</v>
-      </c>
-      <c r="F8" t="s">
-        <v>247</v>
-      </c>
-      <c r="G8" t="s">
-        <v>318</v>
-      </c>
+      <c r="A8" s="6"/>
+      <c r="B8" s="6"/>
+      <c r="C8"/>
+      <c r="D8"/>
+      <c r="E8"/>
+      <c r="F8"/>
+      <c r="G8"/>
     </row>
     <row r="9" ht="32" customHeight="1">
-      <c r="A9" s="6" t="s">
-        <v>31</v>
-      </c>
-      <c r="B9" s="6" t="s">
-        <v>42</v>
-      </c>
-      <c r="C9" t="s">
-        <v>12</v>
-      </c>
-      <c r="D9" t="s">
-        <v>10</v>
-      </c>
-      <c r="E9" t="s">
-        <v>9</v>
-      </c>
-      <c r="F9" t="s">
-        <v>248</v>
-      </c>
-      <c r="G9" t="s">
-        <v>318</v>
-      </c>
+      <c r="A9" s="6"/>
+      <c r="B9" s="6"/>
+      <c r="C9"/>
+      <c r="D9"/>
+      <c r="E9"/>
+      <c r="F9"/>
+      <c r="G9"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -4513,8 +5033,8 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="5" orientation="landscape"/>
   <tableParts count="2">
-    <tablePart r:id="rId32"/>
-    <tablePart r:id="rId33"/>
+    <tablePart r:id="rId28"/>
+    <tablePart r:id="rId29"/>
   </tableParts>
 </worksheet>
 </file>
@@ -4556,10 +5076,10 @@
     </row>
     <row r="3" ht="16" customHeight="1">
       <c r="A3" s="6" t="s">
-        <v>99</v>
+        <v>407</v>
       </c>
       <c r="B3" t="s">
-        <v>174</v>
+        <v>347</v>
       </c>
       <c r="C3" t="s">
         <v>43</v>
@@ -4570,10 +5090,10 @@
     </row>
     <row r="4" ht="32" customHeight="1">
       <c r="A4" s="6" t="s">
-        <v>100</v>
+        <v>408</v>
       </c>
       <c r="B4" t="s">
-        <v>175</v>
+        <v>356</v>
       </c>
       <c r="C4" t="s">
         <v>43</v>
@@ -4584,10 +5104,10 @@
     </row>
     <row r="5" ht="32" customHeight="1">
       <c r="A5" s="6" t="s">
-        <v>101</v>
+        <v>409</v>
       </c>
       <c r="B5" t="s">
-        <v>172</v>
+        <v>361</v>
       </c>
       <c r="C5" t="s">
         <v>43</v>
@@ -4598,10 +5118,10 @@
     </row>
     <row r="6" ht="32" customHeight="1">
       <c r="A6" s="6" t="s">
-        <v>102</v>
+        <v>410</v>
       </c>
       <c r="B6" t="s">
-        <v>172</v>
+        <v>361</v>
       </c>
       <c r="C6" t="s">
         <v>43</v>
@@ -4645,73 +5165,31 @@
       </c>
     </row>
     <row r="10" ht="32" customHeight="1">
-      <c r="A10" s="6" t="s">
-        <v>22</v>
-      </c>
-      <c r="B10" s="6" t="s">
-        <v>42</v>
-      </c>
-      <c r="C10" t="s">
-        <v>8</v>
-      </c>
-      <c r="D10" t="s">
-        <v>11</v>
-      </c>
-      <c r="E10" t="s">
-        <v>9</v>
-      </c>
-      <c r="F10" t="s">
-        <v>249</v>
-      </c>
-      <c r="G10" s="6" t="s">
-        <v>323</v>
-      </c>
+      <c r="A10" s="6"/>
+      <c r="B10" s="6"/>
+      <c r="C10"/>
+      <c r="D10"/>
+      <c r="E10"/>
+      <c r="F10"/>
+      <c r="G10" s="6"/>
     </row>
     <row r="11" ht="32" customHeight="1">
-      <c r="A11" s="6" t="s">
-        <v>23</v>
-      </c>
-      <c r="B11" s="6" t="s">
-        <v>196</v>
-      </c>
-      <c r="C11" t="s">
-        <v>12</v>
-      </c>
-      <c r="D11" t="s">
-        <v>9</v>
-      </c>
-      <c r="E11" t="s">
-        <v>9</v>
-      </c>
-      <c r="F11" t="s">
-        <v>250</v>
-      </c>
-      <c r="G11" s="6" t="s">
-        <v>323</v>
-      </c>
+      <c r="A11" s="6"/>
+      <c r="B11" s="6"/>
+      <c r="C11"/>
+      <c r="D11"/>
+      <c r="E11"/>
+      <c r="F11"/>
+      <c r="G11" s="6"/>
     </row>
     <row r="12" ht="32" customHeight="1">
-      <c r="A12" s="6" t="s">
-        <v>24</v>
-      </c>
-      <c r="B12" s="6" t="s">
-        <v>42</v>
-      </c>
-      <c r="C12" t="s">
-        <v>7</v>
-      </c>
-      <c r="D12" t="s">
-        <v>10</v>
-      </c>
-      <c r="E12" t="s">
-        <v>9</v>
-      </c>
-      <c r="F12" t="s">
-        <v>251</v>
-      </c>
-      <c r="G12" s="6" t="s">
-        <v>323</v>
-      </c>
+      <c r="A12" s="6"/>
+      <c r="B12" s="6"/>
+      <c r="C12"/>
+      <c r="D12"/>
+      <c r="E12"/>
+      <c r="F12"/>
+      <c r="G12" s="6"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -4735,9 +5213,251 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="5" orientation="landscape"/>
   <tableParts count="2">
-    <tablePart r:id="rId34"/>
-    <tablePart r:id="rId35"/>
+    <tablePart r:id="rId30"/>
+    <tablePart r:id="rId31"/>
   </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="s">
+        <v>624</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="s">
+        <v>625</v>
+      </c>
+      <c r="B2" t="s">
+        <v>626</v>
+      </c>
+      <c r="C2" t="s">
+        <v>627</v>
+      </c>
+      <c r="D2" t="s">
+        <v>628</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="s">
+        <v>629</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="s">
+        <v>630</v>
+      </c>
+      <c r="B4" t="s">
+        <v>631</v>
+      </c>
+      <c r="C4" t="s">
+        <v>632</v>
+      </c>
+      <c r="D4" t="s">
+        <v>633</v>
+      </c>
+      <c r="E4" t="s">
+        <v>634</v>
+      </c>
+      <c r="F4" t="s">
+        <v>635</v>
+      </c>
+      <c r="G4" t="s">
+        <v>624</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="s">
+        <v>667</v>
+      </c>
+      <c r="B5" t="s">
+        <v>450</v>
+      </c>
+      <c r="C5" t="s">
+        <v>653</v>
+      </c>
+      <c r="D5" t="s">
+        <v>654</v>
+      </c>
+      <c r="E5" t="s">
+        <v>665</v>
+      </c>
+      <c r="F5" t="s">
+        <v>668</v>
+      </c>
+      <c r="G5" t="s">
+        <v>669</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="s">
+        <v>670</v>
+      </c>
+      <c r="B6" t="s">
+        <v>450</v>
+      </c>
+      <c r="C6" t="s">
+        <v>653</v>
+      </c>
+      <c r="D6" t="s">
+        <v>654</v>
+      </c>
+      <c r="E6" t="s">
+        <v>671</v>
+      </c>
+      <c r="F6" t="s">
+        <v>672</v>
+      </c>
+      <c r="G6" t="s">
+        <v>673</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="s">
+        <v>674</v>
+      </c>
+      <c r="B7" t="s">
+        <v>450</v>
+      </c>
+      <c r="C7" t="s">
+        <v>653</v>
+      </c>
+      <c r="D7" t="s">
+        <v>654</v>
+      </c>
+      <c r="E7" t="s">
+        <v>671</v>
+      </c>
+      <c r="F7" t="s">
+        <v>675</v>
+      </c>
+      <c r="G7" t="s">
+        <v>676</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="s">
+        <v>677</v>
+      </c>
+      <c r="B8" t="s">
+        <v>450</v>
+      </c>
+      <c r="C8" t="s">
+        <v>653</v>
+      </c>
+      <c r="D8" t="s">
+        <v>654</v>
+      </c>
+      <c r="E8" t="s">
+        <v>671</v>
+      </c>
+      <c r="F8" t="s">
+        <v>678</v>
+      </c>
+      <c r="G8" t="s">
+        <v>679</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="s">
+        <v>680</v>
+      </c>
+      <c r="B9" t="s">
+        <v>450</v>
+      </c>
+      <c r="C9" t="s">
+        <v>653</v>
+      </c>
+      <c r="D9" t="s">
+        <v>654</v>
+      </c>
+      <c r="E9" t="s">
+        <v>671</v>
+      </c>
+      <c r="F9" t="s">
+        <v>681</v>
+      </c>
+      <c r="G9" t="s">
+        <v>682</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="s">
+        <v>683</v>
+      </c>
+      <c r="B10" t="s">
+        <v>450</v>
+      </c>
+      <c r="C10" t="s">
+        <v>653</v>
+      </c>
+      <c r="D10" t="s">
+        <v>654</v>
+      </c>
+      <c r="E10" t="s">
+        <v>671</v>
+      </c>
+      <c r="F10" t="s">
+        <v>684</v>
+      </c>
+      <c r="G10" t="s">
+        <v>685</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="s">
+        <v>686</v>
+      </c>
+      <c r="B11" t="s">
+        <v>450</v>
+      </c>
+      <c r="C11" t="s">
+        <v>653</v>
+      </c>
+      <c r="D11" t="s">
+        <v>654</v>
+      </c>
+      <c r="E11" t="s">
+        <v>671</v>
+      </c>
+      <c r="F11" t="s">
+        <v>687</v>
+      </c>
+      <c r="G11" t="s">
+        <v>688</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="s">
+        <v>689</v>
+      </c>
+      <c r="B12" t="s">
+        <v>450</v>
+      </c>
+      <c r="C12" t="s">
+        <v>653</v>
+      </c>
+      <c r="D12" t="s">
+        <v>654</v>
+      </c>
+      <c r="E12" t="s">
+        <v>671</v>
+      </c>
+      <c r="F12" t="s">
+        <v>690</v>
+      </c>
+      <c r="G12" t="s">
+        <v>691</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
 </worksheet>
 </file>
 
@@ -4758,138 +5478,138 @@
     </row>
     <row r="3" ht="20" customHeight="1">
       <c r="A3" s="5" t="s">
-        <v>157</v>
+        <v>411</v>
       </c>
       <c r="B3" s="5"/>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>172</v>
+        <v>361</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>170</v>
+        <v>412</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>171</v>
+        <v>370</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>166</v>
+        <v>413</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>173</v>
+        <v>350</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>167</v>
+        <v>414</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>174</v>
+        <v>347</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>168</v>
+        <v>415</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>175</v>
+        <v>356</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>169</v>
+        <v>416</v>
       </c>
     </row>
     <row r="10" ht="20" customHeight="1">
       <c r="A10" s="5" t="s">
-        <v>159</v>
+        <v>417</v>
       </c>
       <c r="B10" s="5"/>
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>11</v>
+        <v>418</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>163</v>
+        <v>419</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>9</v>
+        <v>420</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>164</v>
+        <v>421</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>10</v>
+        <v>422</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>165</v>
+        <v>423</v>
       </c>
     </row>
     <row r="15" ht="20" customHeight="1">
       <c r="A15" s="5" t="s">
-        <v>160</v>
+        <v>424</v>
       </c>
       <c r="B15" s="5"/>
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>7</v>
+        <v>425</v>
       </c>
       <c r="B16" s="4" t="s">
-        <v>150</v>
+        <v>426</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>12</v>
+        <v>427</v>
       </c>
       <c r="B17" s="4" t="s">
-        <v>151</v>
+        <v>428</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>8</v>
+        <v>429</v>
       </c>
       <c r="B18" s="4" t="s">
-        <v>152</v>
+        <v>430</v>
       </c>
     </row>
     <row r="20" ht="20" customHeight="1">
       <c r="A20" s="5" t="s">
-        <v>158</v>
+        <v>431</v>
       </c>
       <c r="B20" s="5"/>
     </row>
     <row r="21">
       <c r="A21" t="s">
-        <v>11</v>
+        <v>432</v>
       </c>
       <c r="B21" s="4" t="s">
-        <v>148</v>
+        <v>433</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="s">
-        <v>9</v>
+        <v>434</v>
       </c>
       <c r="B22" s="4" t="s">
-        <v>149</v>
+        <v>435</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="s">
-        <v>10</v>
+        <v>436</v>
       </c>
       <c r="B23" s="4" t="s">
-        <v>161</v>
+        <v>437</v>
       </c>
     </row>
   </sheetData>
@@ -4902,12 +5622,6 @@
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait"/>
-  <tableParts count="4">
-    <tablePart r:id="rId4"/>
-    <tablePart r:id="rId5"/>
-    <tablePart r:id="rId6"/>
-    <tablePart r:id="rId7"/>
-  </tableParts>
 </worksheet>
 </file>
 
@@ -4921,92 +5635,92 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>1</v>
+        <v>438</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>7</v>
+        <v>425</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>12</v>
+        <v>427</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>8</v>
+        <v>429</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>4</v>
+        <v>439</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>11</v>
+        <v>418</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>9</v>
+        <v>420</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>10</v>
+        <v>422</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>3</v>
+        <v>440</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>11</v>
+        <v>432</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>9</v>
+        <v>434</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>10</v>
+        <v>436</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>2</v>
+        <v>441</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>175</v>
+        <v>356</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>174</v>
+        <v>347</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>173</v>
+        <v>350</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="s">
-        <v>171</v>
+        <v>370</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="s">
-        <v>172</v>
+        <v>361</v>
       </c>
     </row>
   </sheetData>
@@ -5052,10 +5766,10 @@
     </row>
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="7" t="s">
-        <v>70</v>
+        <v>346</v>
       </c>
       <c r="B3" t="s">
-        <v>174</v>
+        <v>347</v>
       </c>
       <c r="C3" t="s">
         <v>43</v>
@@ -5066,10 +5780,10 @@
     </row>
     <row r="4" ht="16" customHeight="1">
       <c r="A4" s="7" t="s">
-        <v>72</v>
+        <v>348</v>
       </c>
       <c r="B4" t="s">
-        <v>174</v>
+        <v>347</v>
       </c>
       <c r="C4" t="s">
         <v>43</v>
@@ -5080,10 +5794,10 @@
     </row>
     <row r="5" ht="32" customHeight="1">
       <c r="A5" s="7" t="s">
-        <v>74</v>
+        <v>349</v>
       </c>
       <c r="B5" t="s">
-        <v>173</v>
+        <v>350</v>
       </c>
       <c r="C5" t="s">
         <v>43</v>
@@ -5127,27 +5841,13 @@
       </c>
     </row>
     <row r="9" ht="32" customHeight="1">
-      <c r="A9" s="7" t="s">
-        <v>332</v>
-      </c>
-      <c r="B9" s="6" t="s">
-        <v>333</v>
-      </c>
-      <c r="C9" t="s">
-        <v>334</v>
-      </c>
-      <c r="D9" t="s">
-        <v>335</v>
-      </c>
-      <c r="E9" t="s">
-        <v>336</v>
-      </c>
-      <c r="F9" t="s">
-        <v>337</v>
-      </c>
-      <c r="G9" t="s">
-        <v>338</v>
-      </c>
+      <c r="A9" s="7"/>
+      <c r="B9" s="6"/>
+      <c r="C9"/>
+      <c r="D9"/>
+      <c r="E9"/>
+      <c r="F9"/>
+      <c r="G9"/>
     </row>
     <row r="10">
       <c r="A10"/>
@@ -5157,6 +5857,60 @@
       <c r="E10"/>
       <c r="F10"/>
       <c r="G10"/>
+    </row>
+    <row r="11">
+      <c r="A11"/>
+      <c r="B11"/>
+      <c r="C11"/>
+      <c r="D11"/>
+      <c r="E11"/>
+      <c r="F11"/>
+      <c r="G11"/>
+    </row>
+    <row r="12">
+      <c r="A12"/>
+      <c r="B12"/>
+      <c r="C12"/>
+      <c r="D12"/>
+      <c r="E12"/>
+      <c r="F12"/>
+      <c r="G12"/>
+    </row>
+    <row r="13">
+      <c r="A13"/>
+      <c r="B13"/>
+      <c r="C13"/>
+      <c r="D13"/>
+      <c r="E13"/>
+      <c r="F13"/>
+      <c r="G13"/>
+    </row>
+    <row r="14">
+      <c r="A14"/>
+      <c r="B14"/>
+      <c r="C14"/>
+      <c r="D14"/>
+      <c r="E14"/>
+      <c r="F14"/>
+      <c r="G14"/>
+    </row>
+    <row r="15">
+      <c r="A15"/>
+      <c r="B15"/>
+      <c r="C15"/>
+      <c r="D15"/>
+      <c r="E15"/>
+      <c r="F15"/>
+      <c r="G15"/>
+    </row>
+    <row r="16">
+      <c r="A16"/>
+      <c r="B16"/>
+      <c r="C16"/>
+      <c r="D16"/>
+      <c r="E16"/>
+      <c r="F16"/>
+      <c r="G16"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -5180,8 +5934,8 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="5" orientation="landscape"/>
   <tableParts count="2">
-    <tablePart r:id="rId8"/>
-    <tablePart r:id="rId9"/>
+    <tablePart r:id="rId4"/>
+    <tablePart r:id="rId5"/>
   </tableParts>
 </worksheet>
 </file>
@@ -5223,10 +5977,10 @@
     </row>
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="6" t="s">
-        <v>76</v>
+        <v>351</v>
       </c>
       <c r="B3" t="s">
-        <v>174</v>
+        <v>347</v>
       </c>
       <c r="C3" t="s">
         <v>43</v>
@@ -5237,10 +5991,10 @@
     </row>
     <row r="4" ht="32" customHeight="1">
       <c r="A4" s="6" t="s">
-        <v>77</v>
+        <v>352</v>
       </c>
       <c r="B4" t="s">
-        <v>173</v>
+        <v>350</v>
       </c>
       <c r="C4" t="s">
         <v>43</v>
@@ -5284,50 +6038,22 @@
       </c>
     </row>
     <row r="8" ht="32" customHeight="1">
-      <c r="A8" s="6" t="s">
-        <v>40</v>
-      </c>
-      <c r="B8" s="6" t="s">
-        <v>42</v>
-      </c>
-      <c r="C8" t="s">
-        <v>8</v>
-      </c>
-      <c r="D8" t="s">
-        <v>10</v>
-      </c>
-      <c r="E8" t="s">
-        <v>9</v>
-      </c>
-      <c r="F8" t="s">
-        <v>200</v>
-      </c>
-      <c r="G8" t="s">
-        <v>254</v>
-      </c>
+      <c r="A8" s="6"/>
+      <c r="B8" s="6"/>
+      <c r="C8"/>
+      <c r="D8"/>
+      <c r="E8"/>
+      <c r="F8"/>
+      <c r="G8"/>
     </row>
     <row r="9" ht="16" customHeight="1">
-      <c r="A9" s="6" t="s">
-        <v>177</v>
-      </c>
-      <c r="B9" s="6" t="s">
-        <v>194</v>
-      </c>
-      <c r="C9" t="s">
-        <v>12</v>
-      </c>
-      <c r="D9" t="s">
-        <v>11</v>
-      </c>
-      <c r="E9" t="s">
-        <v>9</v>
-      </c>
-      <c r="F9" t="s">
-        <v>201</v>
-      </c>
-      <c r="G9" t="s">
-        <v>254</v>
-      </c>
+      <c r="A9" s="6"/>
+      <c r="B9" s="6"/>
+      <c r="C9"/>
+      <c r="D9"/>
+      <c r="E9"/>
+      <c r="F9"/>
+      <c r="G9"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -5351,8 +6077,8 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="5" orientation="landscape"/>
   <tableParts count="2">
-    <tablePart r:id="rId10"/>
-    <tablePart r:id="rId11"/>
+    <tablePart r:id="rId6"/>
+    <tablePart r:id="rId7"/>
   </tableParts>
 </worksheet>
 </file>
@@ -5394,10 +6120,10 @@
     </row>
     <row r="3" ht="16" customHeight="1">
       <c r="A3" s="6" t="s">
-        <v>78</v>
+        <v>353</v>
       </c>
       <c r="B3" t="s">
-        <v>174</v>
+        <v>347</v>
       </c>
       <c r="C3" t="s">
         <v>43</v>
@@ -5408,10 +6134,10 @@
     </row>
     <row r="4" ht="32" customHeight="1">
       <c r="A4" s="6" t="s">
-        <v>79</v>
+        <v>354</v>
       </c>
       <c r="B4" t="s">
-        <v>173</v>
+        <v>350</v>
       </c>
       <c r="C4" t="s">
         <v>43</v>
@@ -5422,10 +6148,10 @@
     </row>
     <row r="5" ht="32" customHeight="1">
       <c r="A5" s="6" t="s">
-        <v>80</v>
+        <v>355</v>
       </c>
       <c r="B5" t="s">
-        <v>175</v>
+        <v>356</v>
       </c>
       <c r="C5" t="s">
         <v>43</v>
@@ -5436,10 +6162,10 @@
     </row>
     <row r="6" ht="32" customHeight="1">
       <c r="A6" s="6" t="s">
-        <v>114</v>
+        <v>357</v>
       </c>
       <c r="B6" t="s">
-        <v>174</v>
+        <v>347</v>
       </c>
       <c r="C6" t="s">
         <v>43</v>
@@ -5483,96 +6209,40 @@
       </c>
     </row>
     <row r="10" ht="32" customHeight="1">
-      <c r="A10" s="6" t="s">
-        <v>192</v>
-      </c>
-      <c r="B10" s="6" t="s">
-        <v>42</v>
-      </c>
-      <c r="C10" t="s">
-        <v>12</v>
-      </c>
-      <c r="D10" t="s">
-        <v>9</v>
-      </c>
-      <c r="E10" t="s">
-        <v>10</v>
-      </c>
-      <c r="F10" t="s">
-        <v>202</v>
-      </c>
-      <c r="G10" t="s">
-        <v>259</v>
-      </c>
+      <c r="A10" s="6"/>
+      <c r="B10" s="6"/>
+      <c r="C10"/>
+      <c r="D10"/>
+      <c r="E10"/>
+      <c r="F10"/>
+      <c r="G10"/>
     </row>
     <row r="11" ht="32" customHeight="1">
-      <c r="A11" s="6" t="s">
-        <v>30</v>
-      </c>
-      <c r="B11" s="6" t="s">
-        <v>42</v>
-      </c>
-      <c r="C11" t="s">
-        <v>12</v>
-      </c>
-      <c r="D11" t="s">
-        <v>11</v>
-      </c>
-      <c r="E11" t="s">
-        <v>9</v>
-      </c>
-      <c r="F11" t="s">
-        <v>203</v>
-      </c>
-      <c r="G11" t="s">
-        <v>260</v>
-      </c>
+      <c r="A11" s="6"/>
+      <c r="B11" s="6"/>
+      <c r="C11"/>
+      <c r="D11"/>
+      <c r="E11"/>
+      <c r="F11"/>
+      <c r="G11"/>
     </row>
     <row r="12" ht="32" customHeight="1">
-      <c r="A12" s="6" t="s">
-        <v>81</v>
-      </c>
-      <c r="B12" s="6" t="s">
-        <v>42</v>
-      </c>
-      <c r="C12" t="s">
-        <v>12</v>
-      </c>
-      <c r="D12" t="s">
-        <v>10</v>
-      </c>
-      <c r="E12" t="s">
-        <v>9</v>
-      </c>
-      <c r="F12" t="s">
-        <v>204</v>
-      </c>
-      <c r="G12" t="s">
-        <v>259</v>
-      </c>
+      <c r="A12" s="6"/>
+      <c r="B12" s="6"/>
+      <c r="C12"/>
+      <c r="D12"/>
+      <c r="E12"/>
+      <c r="F12"/>
+      <c r="G12"/>
     </row>
     <row r="13" ht="32" customHeight="1">
-      <c r="A13" s="6" t="s">
-        <v>178</v>
-      </c>
-      <c r="B13" s="6" t="s">
-        <v>195</v>
-      </c>
-      <c r="C13" t="s">
-        <v>12</v>
-      </c>
-      <c r="D13" t="s">
-        <v>10</v>
-      </c>
-      <c r="E13" t="s">
-        <v>10</v>
-      </c>
-      <c r="F13" t="s">
-        <v>205</v>
-      </c>
-      <c r="G13" t="s">
-        <v>260</v>
-      </c>
+      <c r="A13" s="6"/>
+      <c r="B13" s="6"/>
+      <c r="C13"/>
+      <c r="D13"/>
+      <c r="E13"/>
+      <c r="F13"/>
+      <c r="G13"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -5596,8 +6266,8 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="5" orientation="landscape"/>
   <tableParts count="2">
-    <tablePart r:id="rId12"/>
-    <tablePart r:id="rId13"/>
+    <tablePart r:id="rId8"/>
+    <tablePart r:id="rId9"/>
   </tableParts>
 </worksheet>
 </file>
@@ -5640,10 +6310,10 @@
     </row>
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="6" t="s">
-        <v>115</v>
+        <v>358</v>
       </c>
       <c r="B3" t="s">
-        <v>174</v>
+        <v>347</v>
       </c>
       <c r="C3" t="s">
         <v>43</v>
@@ -5654,10 +6324,10 @@
     </row>
     <row r="4" ht="32" customHeight="1">
       <c r="A4" s="6" t="s">
-        <v>191</v>
+        <v>359</v>
       </c>
       <c r="B4" t="s">
-        <v>173</v>
+        <v>350</v>
       </c>
       <c r="C4" t="s">
         <v>43</v>
@@ -5668,10 +6338,10 @@
     </row>
     <row r="5" ht="32" customHeight="1">
       <c r="A5" s="6" t="s">
-        <v>82</v>
+        <v>360</v>
       </c>
       <c r="B5" t="s">
-        <v>172</v>
+        <v>361</v>
       </c>
       <c r="C5" t="s">
         <v>43</v>
@@ -5682,10 +6352,10 @@
     </row>
     <row r="6" ht="32" customHeight="1">
       <c r="A6" s="6" t="s">
-        <v>83</v>
+        <v>362</v>
       </c>
       <c r="B6" t="s">
-        <v>172</v>
+        <v>361</v>
       </c>
       <c r="C6" t="s">
         <v>43</v>
@@ -5729,96 +6399,40 @@
       </c>
     </row>
     <row r="10" ht="32" customHeight="1">
-      <c r="A10" s="6" t="s">
-        <v>84</v>
-      </c>
-      <c r="B10" s="6" t="s">
-        <v>193</v>
-      </c>
-      <c r="C10" t="s">
-        <v>8</v>
-      </c>
-      <c r="D10" t="s">
-        <v>10</v>
-      </c>
-      <c r="E10" t="s">
-        <v>10</v>
-      </c>
-      <c r="F10" t="s">
-        <v>206</v>
-      </c>
-      <c r="G10" t="s">
-        <v>265</v>
-      </c>
+      <c r="A10" s="6"/>
+      <c r="B10" s="6"/>
+      <c r="C10"/>
+      <c r="D10"/>
+      <c r="E10"/>
+      <c r="F10"/>
+      <c r="G10"/>
     </row>
     <row r="11" ht="32" customHeight="1">
-      <c r="A11" s="6" t="s">
-        <v>21</v>
-      </c>
-      <c r="B11" s="6" t="s">
-        <v>193</v>
-      </c>
-      <c r="C11" t="s">
-        <v>8</v>
-      </c>
-      <c r="D11" t="s">
-        <v>11</v>
-      </c>
-      <c r="E11" t="s">
-        <v>9</v>
-      </c>
-      <c r="F11" t="s">
-        <v>207</v>
-      </c>
-      <c r="G11" t="s">
-        <v>265</v>
-      </c>
+      <c r="A11" s="6"/>
+      <c r="B11" s="6"/>
+      <c r="C11"/>
+      <c r="D11"/>
+      <c r="E11"/>
+      <c r="F11"/>
+      <c r="G11"/>
     </row>
     <row r="12" ht="32" customHeight="1">
-      <c r="A12" s="6" t="s">
-        <v>20</v>
-      </c>
-      <c r="B12" s="6" t="s">
-        <v>195</v>
-      </c>
-      <c r="C12" t="s">
-        <v>12</v>
-      </c>
-      <c r="D12" t="s">
-        <v>10</v>
-      </c>
-      <c r="E12" t="s">
-        <v>9</v>
-      </c>
-      <c r="F12" t="s">
-        <v>208</v>
-      </c>
-      <c r="G12" t="s">
-        <v>265</v>
-      </c>
+      <c r="A12" s="6"/>
+      <c r="B12" s="6"/>
+      <c r="C12"/>
+      <c r="D12"/>
+      <c r="E12"/>
+      <c r="F12"/>
+      <c r="G12"/>
     </row>
     <row r="13" ht="32" customHeight="1">
-      <c r="A13" s="6" t="s">
-        <v>179</v>
-      </c>
-      <c r="B13" s="6" t="s">
-        <v>42</v>
-      </c>
-      <c r="C13" t="s">
-        <v>12</v>
-      </c>
-      <c r="D13" t="s">
-        <v>10</v>
-      </c>
-      <c r="E13" t="s">
-        <v>9</v>
-      </c>
-      <c r="F13" t="s">
-        <v>209</v>
-      </c>
-      <c r="G13" t="s">
-        <v>265</v>
-      </c>
+      <c r="A13" s="6"/>
+      <c r="B13" s="6"/>
+      <c r="C13"/>
+      <c r="D13"/>
+      <c r="E13"/>
+      <c r="F13"/>
+      <c r="G13"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -5842,8 +6456,8 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="5" orientation="landscape"/>
   <tableParts count="2">
-    <tablePart r:id="rId14"/>
-    <tablePart r:id="rId15"/>
+    <tablePart r:id="rId10"/>
+    <tablePart r:id="rId11"/>
   </tableParts>
 </worksheet>
 </file>
@@ -5886,10 +6500,10 @@
     </row>
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="11" t="s">
-        <v>105</v>
+        <v>363</v>
       </c>
       <c r="B3" t="s">
-        <v>174</v>
+        <v>347</v>
       </c>
       <c r="C3" t="s">
         <v>43</v>
@@ -5900,10 +6514,10 @@
     </row>
     <row r="4" ht="16" customHeight="1">
       <c r="A4" s="11" t="s">
-        <v>106</v>
+        <v>364</v>
       </c>
       <c r="B4" t="s">
-        <v>172</v>
+        <v>361</v>
       </c>
       <c r="C4" t="s">
         <v>43</v>
@@ -5914,10 +6528,10 @@
     </row>
     <row r="5" ht="16" customHeight="1">
       <c r="A5" s="11" t="s">
-        <v>85</v>
+        <v>365</v>
       </c>
       <c r="B5" t="s">
-        <v>174</v>
+        <v>347</v>
       </c>
       <c r="C5" t="s">
         <v>43</v>
@@ -5928,10 +6542,10 @@
     </row>
     <row r="6" ht="32" customHeight="1">
       <c r="A6" s="11" t="s">
-        <v>86</v>
+        <v>366</v>
       </c>
       <c r="B6" t="s">
-        <v>174</v>
+        <v>347</v>
       </c>
       <c r="C6" t="s">
         <v>43</v>
@@ -5978,73 +6592,31 @@
       </c>
     </row>
     <row r="10" ht="32" customHeight="1">
-      <c r="A10" s="6" t="s">
-        <v>87</v>
-      </c>
-      <c r="B10" s="6" t="s">
-        <v>42</v>
-      </c>
-      <c r="C10" t="s">
-        <v>7</v>
-      </c>
-      <c r="D10" t="s">
-        <v>10</v>
-      </c>
-      <c r="E10" t="s">
-        <v>10</v>
-      </c>
-      <c r="F10" t="s">
-        <v>329</v>
-      </c>
-      <c r="G10" t="s">
-        <v>270</v>
-      </c>
+      <c r="A10" s="6"/>
+      <c r="B10" s="6"/>
+      <c r="C10"/>
+      <c r="D10"/>
+      <c r="E10"/>
+      <c r="F10"/>
+      <c r="G10"/>
     </row>
     <row r="11" ht="32" customHeight="1">
-      <c r="A11" s="6" t="s">
-        <v>88</v>
-      </c>
-      <c r="B11" s="6" t="s">
-        <v>42</v>
-      </c>
-      <c r="C11" t="s">
-        <v>12</v>
-      </c>
-      <c r="D11" t="s">
-        <v>10</v>
-      </c>
-      <c r="E11" t="s">
-        <v>10</v>
-      </c>
-      <c r="F11" t="s">
-        <v>330</v>
-      </c>
-      <c r="G11" t="s">
-        <v>270</v>
-      </c>
+      <c r="A11" s="6"/>
+      <c r="B11" s="6"/>
+      <c r="C11"/>
+      <c r="D11"/>
+      <c r="E11"/>
+      <c r="F11"/>
+      <c r="G11"/>
     </row>
     <row r="12" ht="32" customHeight="1">
-      <c r="A12" s="6" t="s">
-        <v>89</v>
-      </c>
-      <c r="B12" s="6" t="s">
-        <v>42</v>
-      </c>
-      <c r="C12" t="s">
-        <v>8</v>
-      </c>
-      <c r="D12" t="s">
-        <v>9</v>
-      </c>
-      <c r="E12" t="s">
-        <v>10</v>
-      </c>
-      <c r="F12" t="s">
-        <v>331</v>
-      </c>
-      <c r="G12" t="s">
-        <v>270</v>
-      </c>
+      <c r="A12" s="6"/>
+      <c r="B12" s="6"/>
+      <c r="C12"/>
+      <c r="D12"/>
+      <c r="E12"/>
+      <c r="F12"/>
+      <c r="G12"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -6068,8 +6640,8 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="5" orientation="landscape"/>
   <tableParts count="2">
-    <tablePart r:id="rId16"/>
-    <tablePart r:id="rId17"/>
+    <tablePart r:id="rId12"/>
+    <tablePart r:id="rId13"/>
   </tableParts>
 </worksheet>
 </file>
@@ -6110,10 +6682,10 @@
     </row>
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="7" t="s">
-        <v>69</v>
+        <v>367</v>
       </c>
       <c r="B3" t="s">
-        <v>172</v>
+        <v>361</v>
       </c>
       <c r="C3" t="s">
         <v>43</v>
@@ -6124,10 +6696,10 @@
     </row>
     <row r="4" ht="16" customHeight="1">
       <c r="A4" s="7" t="s">
-        <v>71</v>
+        <v>368</v>
       </c>
       <c r="B4" t="s">
-        <v>174</v>
+        <v>347</v>
       </c>
       <c r="C4" t="s">
         <v>43</v>
@@ -6138,10 +6710,10 @@
     </row>
     <row r="5" ht="16" customHeight="1">
       <c r="A5" s="7" t="s">
-        <v>73</v>
+        <v>369</v>
       </c>
       <c r="B5" t="s">
-        <v>171</v>
+        <v>370</v>
       </c>
       <c r="C5" t="s">
         <v>43</v>
@@ -6152,10 +6724,10 @@
     </row>
     <row r="6" ht="32" customHeight="1">
       <c r="A6" s="7" t="s">
-        <v>75</v>
+        <v>371</v>
       </c>
       <c r="B6" t="s">
-        <v>175</v>
+        <v>356</v>
       </c>
       <c r="C6" t="s">
         <v>43</v>
@@ -6166,10 +6738,10 @@
     </row>
     <row r="7" ht="16" customHeight="1">
       <c r="A7" s="7" t="s">
-        <v>117</v>
+        <v>372</v>
       </c>
       <c r="B7" t="s">
-        <v>171</v>
+        <v>370</v>
       </c>
       <c r="C7" t="s">
         <v>43</v>
@@ -6180,10 +6752,10 @@
     </row>
     <row r="8" ht="32" customHeight="1">
       <c r="A8" s="7" t="s">
-        <v>91</v>
+        <v>373</v>
       </c>
       <c r="B8" t="s">
-        <v>171</v>
+        <v>370</v>
       </c>
       <c r="C8" s="12" t="s">
         <v>43</v>
@@ -6194,10 +6766,10 @@
     </row>
     <row r="9" ht="32" customHeight="1">
       <c r="A9" s="7" t="s">
-        <v>92</v>
+        <v>374</v>
       </c>
       <c r="B9" t="s">
-        <v>174</v>
+        <v>347</v>
       </c>
       <c r="C9" s="12" t="s">
         <v>43</v>
@@ -6208,10 +6780,10 @@
     </row>
     <row r="10" ht="32" customHeight="1">
       <c r="A10" s="7" t="s">
-        <v>93</v>
+        <v>375</v>
       </c>
       <c r="B10" t="s">
-        <v>174</v>
+        <v>347</v>
       </c>
       <c r="C10" s="12" t="s">
         <v>43</v>
@@ -6255,119 +6827,49 @@
       </c>
     </row>
     <row r="14" ht="32" customHeight="1">
-      <c r="A14" s="7" t="s">
-        <v>188</v>
-      </c>
-      <c r="B14" s="6" t="s">
-        <v>193</v>
-      </c>
-      <c r="C14" t="s">
-        <v>7</v>
-      </c>
-      <c r="D14" t="s">
-        <v>9</v>
-      </c>
-      <c r="E14" t="s">
-        <v>9</v>
-      </c>
-      <c r="F14" t="s">
-        <v>210</v>
-      </c>
-      <c r="G14" s="6" t="s">
-        <v>279</v>
-      </c>
+      <c r="A14" s="7"/>
+      <c r="B14" s="6"/>
+      <c r="C14"/>
+      <c r="D14"/>
+      <c r="E14"/>
+      <c r="F14"/>
+      <c r="G14" s="6"/>
     </row>
     <row r="15" ht="32" customHeight="1">
-      <c r="A15" s="7" t="s">
-        <v>187</v>
-      </c>
-      <c r="B15" s="6" t="s">
-        <v>193</v>
-      </c>
-      <c r="C15" t="s">
-        <v>7</v>
-      </c>
-      <c r="D15" t="s">
-        <v>9</v>
-      </c>
-      <c r="E15" t="s">
-        <v>9</v>
-      </c>
-      <c r="F15" t="s">
-        <v>211</v>
-      </c>
-      <c r="G15" s="6" t="s">
-        <v>279</v>
-      </c>
+      <c r="A15" s="7"/>
+      <c r="B15" s="6"/>
+      <c r="C15"/>
+      <c r="D15"/>
+      <c r="E15"/>
+      <c r="F15"/>
+      <c r="G15" s="6"/>
     </row>
     <row r="16" ht="32" customHeight="1">
-      <c r="A16" s="7" t="s">
-        <v>189</v>
-      </c>
-      <c r="B16" s="6" t="s">
-        <v>193</v>
-      </c>
-      <c r="C16" t="s">
-        <v>12</v>
-      </c>
-      <c r="D16" t="s">
-        <v>9</v>
-      </c>
-      <c r="E16" t="s">
-        <v>9</v>
-      </c>
-      <c r="F16" t="s">
-        <v>212</v>
-      </c>
-      <c r="G16" s="6" t="s">
-        <v>279</v>
-      </c>
+      <c r="A16" s="7"/>
+      <c r="B16" s="6"/>
+      <c r="C16"/>
+      <c r="D16"/>
+      <c r="E16"/>
+      <c r="F16"/>
+      <c r="G16" s="6"/>
     </row>
     <row r="17" ht="32" customHeight="1">
-      <c r="A17" s="7" t="s">
-        <v>16</v>
-      </c>
-      <c r="B17" s="6" t="s">
-        <v>193</v>
-      </c>
-      <c r="C17" t="s">
-        <v>12</v>
-      </c>
-      <c r="D17" t="s">
-        <v>9</v>
-      </c>
-      <c r="E17" t="s">
-        <v>9</v>
-      </c>
-      <c r="F17" t="s">
-        <v>213</v>
-      </c>
-      <c r="G17" s="6" t="s">
-        <v>324</v>
-      </c>
+      <c r="A17" s="7"/>
+      <c r="B17" s="6"/>
+      <c r="C17"/>
+      <c r="D17"/>
+      <c r="E17"/>
+      <c r="F17"/>
+      <c r="G17" s="6"/>
     </row>
     <row r="18" ht="32" customHeight="1">
-      <c r="A18" s="7" t="s">
-        <v>190</v>
-      </c>
-      <c r="B18" s="6" t="s">
-        <v>193</v>
-      </c>
-      <c r="C18" t="s">
-        <v>12</v>
-      </c>
-      <c r="D18" t="s">
-        <v>9</v>
-      </c>
-      <c r="E18" t="s">
-        <v>10</v>
-      </c>
-      <c r="F18" t="s">
-        <v>214</v>
-      </c>
-      <c r="G18" s="6" t="s">
-        <v>280</v>
-      </c>
+      <c r="A18" s="7"/>
+      <c r="B18" s="6"/>
+      <c r="C18"/>
+      <c r="D18"/>
+      <c r="E18"/>
+      <c r="F18"/>
+      <c r="G18" s="6"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -6391,8 +6893,8 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="5" orientation="landscape"/>
   <tableParts count="2">
-    <tablePart r:id="rId18"/>
-    <tablePart r:id="rId19"/>
+    <tablePart r:id="rId14"/>
+    <tablePart r:id="rId15"/>
   </tableParts>
 </worksheet>
 </file>
</xml_diff>